<commit_message>
Layout on the cleared block
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -1324,7 +1324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>748:470</t>
+          <t>744:464</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>Trap 1 site 743:462; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H20" s="4" t="n"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>750:478</t>
+          <t>744:480</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>Trap 2 site 743:478; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H21" s="4" t="n"/>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>745:461</t>
+          <t>746:454</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Trap 1 site 743:462; 4 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H22" s="4" t="n"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>745:477</t>
+          <t>745:461</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Trap 2 site 743:478; 5 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H23" s="4" t="n"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>750:458</t>
+          <t>745:477</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H24" s="4" t="n"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>744:464</t>
+          <t>748:470</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H25" s="4" t="n"/>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>748:454</t>
+          <t>750:478</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H26" s="4" t="n"/>
@@ -2188,35 +2188,35 @@
       <c r="J26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>743:480</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>5 slots (file order)</t>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>750:458</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H27" s="4" t="n"/>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>742:480</t>
+          <t>739:458</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -2243,14 +2243,18 @@
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
           <t>wave 1 complete</t>
         </is>
       </c>
-      <c r="G28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>9 slots (file order)</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -2266,7 +2270,7 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>742:464</t>
+          <t>739:474</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -2275,7 +2279,7 @@
         </is>
       </c>
       <c r="E29" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
@@ -2284,7 +2288,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H29" s="4" t="n"/>
@@ -2302,7 +2306,7 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>741:470</t>
+          <t>743:470</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -2311,7 +2315,7 @@
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
@@ -2320,7 +2324,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>11 slots (file order)</t>
+          <t>9 slots (file order)</t>
         </is>
       </c>
       <c r="H30" s="4" t="n"/>
@@ -2338,7 +2342,7 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>742:454</t>
+          <t>742:487</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -2356,7 +2360,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H31" s="4" t="n"/>
@@ -2374,7 +2378,7 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>739:458</t>
+          <t>742:480</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -2392,7 +2396,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H32" s="4" t="n"/>
@@ -2410,7 +2414,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>739:474</t>
+          <t>748:485</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -2428,7 +2432,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>6 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H33" s="4" t="n"/>
@@ -2446,7 +2450,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>748:485</t>
+          <t>742:464</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -2464,7 +2468,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H34" s="4" t="n"/>
@@ -2472,35 +2476,35 @@
       <c r="J34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n">
+      <c r="A35" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>741:487</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="n">
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>739:451</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>6 slots (file order)</t>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H35" s="4" t="n"/>
@@ -2518,7 +2522,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>735:481</t>
+          <t>735:465</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
@@ -2554,7 +2558,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>735:467</t>
+          <t>736:469</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -2572,7 +2576,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H37" s="4" t="n"/>
@@ -2590,7 +2594,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>735:460</t>
+          <t>732:458</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -2608,7 +2612,7 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>6 slots (file order)</t>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H38" s="4" t="n"/>
@@ -2626,7 +2630,7 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>732:474</t>
+          <t>735:483</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2644,7 +2648,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H39" s="4" t="n"/>
@@ -2652,33 +2656,35 @@
       <c r="J39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n">
+      <c r="A40" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D40" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="inlineStr"/>
-      <c r="F40" s="10" t="inlineStr">
-        <is>
-          <t>banner 745:461 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G40" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 11</t>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>735:476</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>wave 3</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>wave 2 complete</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>6 slots (file order)</t>
         </is>
       </c>
       <c r="H40" s="4" t="n"/>
@@ -2691,12 +2697,12 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>743:478</t>
+          <t>743:462</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -2707,17 +2713,51 @@
       <c r="E41" s="10" t="inlineStr"/>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>banner 745:477 (wave 1); the old trap's last firing</t>
+          <t>banner 744:464 (wave 1); the old trap's last firing</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>ring 1 seats: 11</t>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr"/>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>banner 744:480 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2804,28 +2844,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>740:461</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="8" t="n">
+      <c r="A2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>742:459</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="8" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="G2" s="8" t="n">
-        <v>2</v>
+      <c r="F2" s="7" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
@@ -2833,28 +2873,28 @@
       <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>744:459</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>1</v>
+      <c r="A3" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>740:461</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
@@ -2862,28 +2902,28 @@
       <c r="K3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>740:463</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="8" t="n">
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>744:459</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="8" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>2</v>
+      <c r="F4" s="7" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
@@ -2891,28 +2931,28 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>746:461</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>1</v>
+      <c r="A5" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>740:463</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
@@ -2921,11 +2961,11 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>742:465</t>
+          <t>746:461</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -2938,7 +2978,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>13</v>
+        <v>11.3</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>1</v>
@@ -2949,28 +2989,28 @@
       <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>740:459</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="8" t="n">
+      <c r="A7" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>742:465</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F7" s="8" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>2</v>
+      <c r="F7" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
@@ -2978,28 +3018,28 @@
       <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>746:463</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>1</v>
+      <c r="A8" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>740:459</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
@@ -3012,7 +3052,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>744:465</t>
+          <t>746:463</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
@@ -3025,7 +3065,7 @@
         <v>14</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>11.1</v>
+        <v>10.1</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>1</v>
@@ -3037,11 +3077,11 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>746:459</t>
+          <t>744:465</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -3051,10 +3091,10 @@
         <v>1</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>12.7</v>
+        <v>11.1</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>1</v>
@@ -3065,28 +3105,28 @@
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>740:465</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="8" t="n">
+      <c r="A11" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>746:459</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="8" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>2</v>
+      <c r="F11" s="7" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
@@ -3094,28 +3134,28 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>746:465</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>1</v>
+      <c r="A12" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>740:465</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
@@ -3123,28 +3163,28 @@
       <c r="K12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>742:457</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>2</v>
+      <c r="A13" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>746:465</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
@@ -3152,28 +3192,28 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>738:461</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="9" t="n">
+      <c r="A14" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>742:457</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="9" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>3</v>
+      <c r="F14" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
@@ -3181,28 +3221,28 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>744:457</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>2</v>
+      <c r="A15" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>738:461</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -3210,28 +3250,28 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>738:463</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="9" t="n">
+      <c r="A16" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>744:457</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="F16" s="9" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>3</v>
+      <c r="F16" s="7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -3239,28 +3279,28 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n">
-        <v>33</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>740:457</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>2</v>
+      <c r="A17" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>738:463</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -3269,11 +3309,11 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>738:459</t>
+          <t>740:457</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
@@ -3286,7 +3326,7 @@
         <v>17</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>19</v>
+        <v>18.5</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>2</v>
@@ -3297,28 +3337,28 @@
       <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>748:461</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>1</v>
+      <c r="A19" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>738:459</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
@@ -3326,28 +3366,28 @@
       <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n">
+      <c r="A20" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>742:467</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="8" t="n">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>748:461</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="8" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G20" s="8" t="n">
-        <v>2</v>
+      <c r="F20" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -3355,28 +3395,28 @@
       <c r="K20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>748:463</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="6" t="n">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>742:467</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F21" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>0</v>
+      <c r="F21" s="8" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
@@ -3384,28 +3424,28 @@
       <c r="K21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n">
+      <c r="A22" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>744:467</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="8" t="n">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>748:463</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="8" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>2</v>
+      <c r="F22" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
@@ -3413,28 +3453,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>746:457</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="7" t="n">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>744:467</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="7" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>1</v>
+      <c r="F23" s="8" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -3442,28 +3482,28 @@
       <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>738:465</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="9" t="n">
+      <c r="A24" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>746:457</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F24" s="9" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>3</v>
+      <c r="F24" s="7" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -3471,28 +3511,28 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n">
-        <v>48</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>748:459</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>1</v>
+      <c r="A25" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>738:465</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -3500,28 +3540,28 @@
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
-        <v>49</v>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>740:467</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="8" t="n">
+      <c r="A26" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>748:459</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="F26" s="8" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G26" s="8" t="n">
-        <v>2</v>
+      <c r="F26" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
@@ -3529,28 +3569,28 @@
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>748:465</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>0</v>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>740:467</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -3558,28 +3598,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>746:467</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="7" t="n">
+      <c r="A28" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>748:465</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="7" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <v>1</v>
+      <c r="F28" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -3588,11 +3628,11 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>748:457</t>
+          <t>746:467</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
@@ -3602,10 +3642,10 @@
         <v>2</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>13.2</v>
+        <v>8.6</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>1</v>
@@ -3616,28 +3656,28 @@
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="n">
-        <v>68</v>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>738:467</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="8" t="n">
+      <c r="A30" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>748:457</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F30" s="8" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="G30" s="8" t="n">
-        <v>2</v>
+      <c r="F30" s="7" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
@@ -3645,28 +3685,28 @@
       <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
-        <v>77</v>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>748:467</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F31" s="6" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G31" s="6" t="n">
-        <v>0</v>
+      <c r="A31" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>738:467</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
@@ -3674,28 +3714,28 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>742:455</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="G32" s="8" t="n">
-        <v>2</v>
+      <c r="A32" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>748:467</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -3703,28 +3743,28 @@
       <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="n">
-        <v>57</v>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>736:461</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="9" t="n">
+      <c r="A33" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>742:455</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="9" t="n">
+      <c r="E33" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F33" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <v>3</v>
+      <c r="F33" s="8" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -3732,28 +3772,28 @@
       <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="9" t="n">
         <v>59</v>
       </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>744:455</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="8" t="n">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>736:461</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E34" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F34" s="8" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="G34" s="8" t="n">
-        <v>2</v>
+      <c r="E34" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
@@ -3761,28 +3801,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>736:463</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="9" t="n">
+      <c r="A35" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>744:455</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="9" t="n">
+      <c r="E35" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F35" s="9" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G35" s="9" t="n">
-        <v>3</v>
+      <c r="F35" s="7" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -3790,28 +3830,28 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="n">
-        <v>64</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>740:455</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="8" t="n">
+      <c r="A36" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>736:463</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="E36" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="F36" s="8" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G36" s="8" t="n">
-        <v>2</v>
+      <c r="F36" s="9" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
@@ -3820,11 +3860,11 @@
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>736:459</t>
+          <t>740:455</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
@@ -3837,7 +3877,7 @@
         <v>21</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>20.8</v>
+        <v>19.8</v>
       </c>
       <c r="G37" s="8" t="n">
         <v>2</v>
@@ -3848,28 +3888,28 @@
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>746:455</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="7" t="n">
+      <c r="A38" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>736:459</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="F38" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="G38" s="7" t="n">
-        <v>1</v>
+      <c r="E38" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
@@ -3877,28 +3917,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="n">
-        <v>72</v>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>736:465</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="9" t="n">
+      <c r="A39" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>746:455</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="9" t="n">
+      <c r="E39" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F39" s="9" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <v>3</v>
+      <c r="F39" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -3906,28 +3946,28 @@
       <c r="K39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>742:469</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="8" t="n">
+      <c r="A40" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>736:465</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E40" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="F40" s="8" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G40" s="8" t="n">
-        <v>2</v>
+      <c r="E40" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
@@ -3936,7 +3976,7 @@
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
@@ -3965,7 +4005,7 @@
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
@@ -3994,7 +4034,7 @@
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
@@ -4022,28 +4062,28 @@
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
-        <v>83</v>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>746:469</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="7" t="n">
+      <c r="A44" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>740:469</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="F44" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G44" s="7" t="n">
-        <v>1</v>
+      <c r="E44" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
@@ -4052,11 +4092,11 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>748:455</t>
+          <t>746:469</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
@@ -4069,7 +4109,7 @@
         <v>25</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>15</v>
+        <v>8.5</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>1</v>
@@ -4080,28 +4120,28 @@
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="n">
-        <v>87</v>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>736:467</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="9" t="n">
+      <c r="A46" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>748:455</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="9" t="n">
+      <c r="E46" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F46" s="9" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G46" s="9" t="n">
-        <v>3</v>
+      <c r="F46" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
@@ -4109,28 +4149,28 @@
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>736:455</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="8" t="n">
+      <c r="A47" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>736:467</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>27</v>
-      </c>
-      <c r="F47" s="8" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="G47" s="8" t="n">
-        <v>2</v>
+      <c r="E47" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
@@ -4139,24 +4179,24 @@
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>734:461</t>
+          <t>738:469</t>
         </is>
       </c>
       <c r="C48" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D48" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E48" s="9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>21.8</v>
+        <v>16.5</v>
       </c>
       <c r="G48" s="9" t="n">
         <v>3</v>
@@ -4168,11 +4208,11 @@
     </row>
     <row r="49">
       <c r="A49" s="8" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>744:453</t>
+          <t>742:453</t>
         </is>
       </c>
       <c r="C49" s="8" t="n">
@@ -4182,10 +4222,10 @@
         <v>4</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>18.7</v>
+        <v>19.9</v>
       </c>
       <c r="G49" s="8" t="n">
         <v>2</v>
@@ -4197,11 +4237,11 @@
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>734:463</t>
+          <t>734:461</t>
         </is>
       </c>
       <c r="C50" s="9" t="n">
@@ -4211,10 +4251,10 @@
         <v>4</v>
       </c>
       <c r="E50" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>21.2</v>
+        <v>21.8</v>
       </c>
       <c r="G50" s="9" t="n">
         <v>3</v>
@@ -4225,28 +4265,28 @@
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>740:453</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="8" t="n">
+      <c r="A51" s="7" t="n">
+        <v>97</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>744:453</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E51" s="8" t="n">
+      <c r="E51" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="F51" s="8" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="G51" s="8" t="n">
-        <v>2</v>
+      <c r="F51" s="7" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
@@ -4254,28 +4294,28 @@
       <c r="K51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="n">
-        <v>97</v>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>746:453</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="7" t="n">
+      <c r="A52" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>734:463</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="F52" s="7" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>1</v>
+      <c r="E52" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
@@ -4283,28 +4323,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
-        <v>99</v>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>734:465</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E53" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="F53" s="9" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <v>3</v>
+      <c r="A53" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>742:475</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F53" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G53" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4312,28 +4352,28 @@
       <c r="K53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>742:475</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="7" t="n">
+      <c r="A54" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>740:477</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F54" s="7" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="G54" s="7" t="n">
-        <v>1</v>
+      <c r="F54" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
@@ -4341,28 +4381,28 @@
       <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>740:477</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F55" s="8" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="G55" s="8" t="n">
-        <v>2</v>
+      <c r="A55" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>744:475</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -4370,28 +4410,28 @@
       <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>744:475</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="7" t="n">
+      <c r="A56" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>740:479</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="F56" s="7" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="G56" s="7" t="n">
-        <v>1</v>
+      <c r="F56" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
@@ -4399,28 +4439,28 @@
       <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>740:479</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="F57" s="8" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G57" s="8" t="n">
-        <v>2</v>
+      <c r="A57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>746:477</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F57" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -4428,28 +4468,28 @@
       <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>746:477</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="7" t="n">
+      <c r="A58" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>740:475</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F58" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="G58" s="7" t="n">
-        <v>1</v>
+      <c r="F58" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
@@ -4457,28 +4497,28 @@
       <c r="K58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>740:475</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="8" t="n">
+      <c r="A59" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>742:481</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F59" s="8" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="G59" s="8" t="n">
-        <v>2</v>
+      <c r="F59" s="7" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G59" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H59" s="4" t="n"/>
       <c r="I59" s="4" t="n"/>
@@ -4486,28 +4526,28 @@
       <c r="K59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>742:481</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="F60" s="8" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G60" s="8" t="n">
-        <v>2</v>
+      <c r="A60" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>746:479</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F60" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G60" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
@@ -4515,28 +4555,28 @@
       <c r="K60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="A61" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>744:481</t>
         </is>
       </c>
-      <c r="C61" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D61" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="8" t="n">
+      <c r="C61" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="F61" s="8" t="n">
+      <c r="F61" s="7" t="n">
         <v>16.3</v>
       </c>
-      <c r="G61" s="8" t="n">
-        <v>2</v>
+      <c r="G61" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
@@ -4545,7 +4585,7 @@
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
@@ -4574,7 +4614,7 @@
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
@@ -4602,28 +4642,28 @@
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="A64" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>746:481</t>
         </is>
       </c>
-      <c r="C64" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="8" t="n">
+      <c r="C64" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="F64" s="8" t="n">
+      <c r="F64" s="7" t="n">
         <v>15.1</v>
       </c>
-      <c r="G64" s="8" t="n">
-        <v>2</v>
+      <c r="G64" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
@@ -4632,7 +4672,7 @@
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
@@ -4661,7 +4701,7 @@
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
@@ -4690,7 +4730,7 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
@@ -4719,7 +4759,7 @@
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
@@ -4748,7 +4788,7 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
@@ -4777,7 +4817,7 @@
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
@@ -4806,7 +4846,7 @@
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
@@ -4834,28 +4874,28 @@
       <c r="K71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B72" s="9" t="inlineStr">
+      <c r="A72" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>742:483</t>
         </is>
       </c>
-      <c r="C72" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" s="9" t="n">
+      <c r="C72" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F72" s="9" t="n">
+      <c r="F72" s="8" t="n">
         <v>19.1</v>
       </c>
-      <c r="G72" s="9" t="n">
-        <v>3</v>
+      <c r="G72" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
@@ -4864,7 +4904,7 @@
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
@@ -4893,7 +4933,7 @@
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
@@ -4921,28 +4961,28 @@
       <c r="K74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="B75" s="9" t="inlineStr">
+      <c r="A75" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>744:483</t>
         </is>
       </c>
-      <c r="C75" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D75" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" s="9" t="n">
+      <c r="C75" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F75" s="9" t="n">
+      <c r="F75" s="8" t="n">
         <v>17.9</v>
       </c>
-      <c r="G75" s="9" t="n">
-        <v>3</v>
+      <c r="G75" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
@@ -4951,7 +4991,7 @@
     </row>
     <row r="76">
       <c r="A76" s="9" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
@@ -4980,7 +5020,7 @@
     </row>
     <row r="77">
       <c r="A77" s="6" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
@@ -5008,28 +5048,28 @@
       <c r="K77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="B78" s="9" t="inlineStr">
+      <c r="A78" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>740:483</t>
         </is>
       </c>
-      <c r="C78" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D78" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E78" s="9" t="n">
+      <c r="C78" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="F78" s="9" t="n">
+      <c r="F78" s="8" t="n">
         <v>20.5</v>
       </c>
-      <c r="G78" s="9" t="n">
-        <v>3</v>
+      <c r="G78" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
@@ -5038,7 +5078,7 @@
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
@@ -5067,7 +5107,7 @@
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
@@ -5096,7 +5136,7 @@
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
@@ -5125,7 +5165,7 @@
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
@@ -5154,7 +5194,7 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
@@ -5183,7 +5223,7 @@
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
@@ -5211,28 +5251,28 @@
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="n">
-        <v>58</v>
-      </c>
-      <c r="B85" s="8" t="inlineStr">
-        <is>
-          <t>744:471</t>
-        </is>
-      </c>
-      <c r="C85" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="8" t="n">
+      <c r="A85" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>736:477</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E85" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F85" s="8" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="G85" s="8" t="n">
-        <v>2</v>
+      <c r="E85" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F85" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
@@ -5240,28 +5280,28 @@
       <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="9" t="n">
+      <c r="A86" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="B86" s="9" t="inlineStr">
-        <is>
-          <t>736:479</t>
-        </is>
-      </c>
-      <c r="C86" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="9" t="n">
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>744:471</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E86" s="9" t="n">
+      <c r="E86" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="F86" s="9" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G86" s="9" t="n">
-        <v>3</v>
+      <c r="F86" s="8" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G86" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -5269,28 +5309,28 @@
       <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="n">
-        <v>62</v>
-      </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>740:471</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="8" t="n">
+      <c r="A87" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>736:479</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E87" s="8" t="n">
+      <c r="E87" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="F87" s="8" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="G87" s="8" t="n">
-        <v>2</v>
+      <c r="F87" s="9" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H87" s="4" t="n"/>
       <c r="I87" s="4" t="n"/>
@@ -5299,11 +5339,11 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>736:475</t>
+          <t>740:471</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
@@ -5316,7 +5356,7 @@
         <v>21</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>19.6</v>
+        <v>14.7</v>
       </c>
       <c r="G88" s="8" t="n">
         <v>2</v>
@@ -5327,28 +5367,28 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="B89" s="7" t="inlineStr">
-        <is>
-          <t>746:471</t>
-        </is>
-      </c>
-      <c r="C89" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D89" s="7" t="n">
+      <c r="A89" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>736:475</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E89" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="F89" s="7" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G89" s="7" t="n">
-        <v>1</v>
+      <c r="E89" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F89" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G89" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
@@ -5356,28 +5396,28 @@
       <c r="K89" s="4" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="9" t="n">
+      <c r="A90" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="B90" s="9" t="inlineStr">
-        <is>
-          <t>736:481</t>
-        </is>
-      </c>
-      <c r="C90" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D90" s="9" t="n">
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>746:471</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E90" s="9" t="n">
+      <c r="E90" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F90" s="9" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="G90" s="9" t="n">
-        <v>3</v>
+      <c r="F90" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G90" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H90" s="4" t="n"/>
       <c r="I90" s="4" t="n"/>
@@ -5390,7 +5430,7 @@
       </c>
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>744:485</t>
+          <t>736:481</t>
         </is>
       </c>
       <c r="C91" s="9" t="n">
@@ -5400,10 +5440,10 @@
         <v>3</v>
       </c>
       <c r="E91" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F91" s="9" t="n">
-        <v>19.6</v>
+        <v>22.3</v>
       </c>
       <c r="G91" s="9" t="n">
         <v>3</v>
@@ -5415,11 +5455,11 @@
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>736:473</t>
+          <t>742:485</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
@@ -5429,10 +5469,10 @@
         <v>3</v>
       </c>
       <c r="E92" s="8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>19</v>
+        <v>20.7</v>
       </c>
       <c r="G92" s="8" t="n">
         <v>2</v>
@@ -5443,28 +5483,28 @@
       <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="9" t="n">
-        <v>82</v>
-      </c>
-      <c r="B93" s="9" t="inlineStr">
-        <is>
-          <t>740:485</t>
-        </is>
-      </c>
-      <c r="C93" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="9" t="n">
+      <c r="A93" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>744:485</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E93" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="F93" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="G93" s="9" t="n">
-        <v>3</v>
+      <c r="E93" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="F93" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G93" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H93" s="4" t="n"/>
       <c r="I93" s="4" t="n"/>
@@ -5473,11 +5513,11 @@
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>746:485</t>
+          <t>738:471</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
@@ -5487,10 +5527,10 @@
         <v>3</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>18.6</v>
+        <v>16.7</v>
       </c>
       <c r="G94" s="8" t="n">
         <v>2</v>
@@ -5501,28 +5541,28 @@
       <c r="K94" s="4" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="n">
-        <v>85</v>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>748:471</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D95" s="6" t="n">
+      <c r="A95" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>736:473</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E95" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="F95" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G95" s="6" t="n">
-        <v>0</v>
+      <c r="E95" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F95" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="G95" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H95" s="4" t="n"/>
       <c r="I95" s="4" t="n"/>
@@ -5530,28 +5570,28 @@
       <c r="K95" s="4" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="B96" s="9" t="inlineStr">
-        <is>
-          <t>736:483</t>
-        </is>
-      </c>
-      <c r="C96" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="9" t="n">
+      <c r="A96" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>740:485</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="F96" s="9" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G96" s="9" t="n">
-        <v>3</v>
+      <c r="E96" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F96" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="G96" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H96" s="4" t="n"/>
       <c r="I96" s="4" t="n"/>
@@ -5559,28 +5599,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="9" t="n">
-        <v>94</v>
-      </c>
-      <c r="B97" s="9" t="inlineStr">
-        <is>
-          <t>738:485</t>
-        </is>
-      </c>
-      <c r="C97" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="9" t="n">
+      <c r="A97" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>746:485</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="F97" s="9" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="G97" s="9" t="n">
-        <v>3</v>
+      <c r="E97" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F97" s="8" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G97" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
@@ -5588,28 +5628,28 @@
       <c r="K97" s="4" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="n">
-        <v>98</v>
-      </c>
-      <c r="B98" s="8" t="inlineStr">
-        <is>
-          <t>736:471</t>
-        </is>
-      </c>
-      <c r="C98" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D98" s="8" t="n">
+      <c r="A98" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>748:471</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D98" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E98" s="8" t="n">
-        <v>27</v>
-      </c>
-      <c r="F98" s="8" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G98" s="8" t="n">
-        <v>2</v>
+      <c r="E98" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F98" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G98" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H98" s="4" t="n"/>
       <c r="I98" s="4" t="n"/>
@@ -5618,24 +5658,24 @@
     </row>
     <row r="99">
       <c r="A99" s="9" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>734:477</t>
+          <t>736:483</t>
         </is>
       </c>
       <c r="C99" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D99" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E99" s="9" t="n">
         <v>25</v>
       </c>
       <c r="F99" s="9" t="n">
-        <v>22.2</v>
+        <v>23.5</v>
       </c>
       <c r="G99" s="9" t="n">
         <v>3</v>
@@ -5647,11 +5687,11 @@
     </row>
     <row r="100">
       <c r="A100" s="9" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>734:479</t>
+          <t>734:477</t>
         </is>
       </c>
       <c r="C100" s="9" t="n">
@@ -5661,10 +5701,10 @@
         <v>4</v>
       </c>
       <c r="E100" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F100" s="9" t="n">
-        <v>23</v>
+        <v>22.2</v>
       </c>
       <c r="G100" s="9" t="n">
         <v>3</v>
@@ -5676,11 +5716,11 @@
     </row>
     <row r="101">
       <c r="A101" s="9" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>734:475</t>
+          <t>734:479</t>
         </is>
       </c>
       <c r="C101" s="9" t="n">
@@ -5693,7 +5733,7 @@
         <v>26</v>
       </c>
       <c r="F101" s="9" t="n">
-        <v>21.5</v>
+        <v>23</v>
       </c>
       <c r="G101" s="9" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Seats on both sides of the Fertile line
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -1324,7 +1324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>746:454</t>
+          <t>745:461</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H22" s="4" t="n"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>745:461</t>
+          <t>745:477</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H23" s="4" t="n"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>745:477</t>
+          <t>752:480</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H24" s="4" t="n"/>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>750:478</t>
+          <t>750:458</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H26" s="4" t="n"/>
@@ -2188,35 +2188,35 @@
       <c r="J26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>750:458</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="n">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>739:458</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>3 slots (file order)</t>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H27" s="4" t="n"/>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>739:458</t>
+          <t>739:474</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>9 slots (file order)</t>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H28" s="4" t="n"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>739:474</t>
+          <t>743:470</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>9 slots (file order)</t>
         </is>
       </c>
       <c r="H29" s="4" t="n"/>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>743:470</t>
+          <t>737:483</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>9 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H30" s="4" t="n"/>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>742:487</t>
+          <t>744:487</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H31" s="4" t="n"/>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>742:480</t>
+          <t>742:464</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H32" s="4" t="n"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>748:485</t>
+          <t>750:483</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H33" s="4" t="n"/>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>742:464</t>
+          <t>742:480</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H34" s="4" t="n"/>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>739:451</t>
+          <t>744:454</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>1 slots (file order)</t>
+          <t>6 slots (file order)</t>
         </is>
       </c>
       <c r="H35" s="4" t="n"/>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>8 slots (file order)</t>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H36" s="4" t="n"/>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>736:469</t>
+          <t>735:476</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H37" s="4" t="n"/>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>732:458</t>
+          <t>736:469</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -2620,35 +2620,33 @@
       <c r="J38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="n">
+      <c r="A39" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>735:483</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>4 slots (file order)</t>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr"/>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>banner 744:464 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H39" s="4" t="n"/>
@@ -2656,108 +2654,38 @@
       <c r="J39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="n">
+      <c r="A40" s="10" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>735:476</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="F40" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>6 slots (file order)</t>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr"/>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>banner 744:480 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
       <c r="J40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E41" s="10" t="inlineStr"/>
-      <c r="F41" s="10" t="inlineStr">
-        <is>
-          <t>banner 744:464 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G41" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E42" s="10" t="inlineStr"/>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>banner 744:480 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G42" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3250,28 +3178,28 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>744:457</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="7" t="n">
+      <c r="C16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="8" t="n">
         <v>15.6</v>
       </c>
-      <c r="G16" s="7" t="n">
-        <v>1</v>
+      <c r="G16" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -3482,28 +3410,28 @@
       <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>746:457</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="7" t="n">
+      <c r="C24" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F24" s="7" t="n">
+      <c r="F24" s="8" t="n">
         <v>14.3</v>
       </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
+      <c r="G24" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -3715,7 +3643,7 @@
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
@@ -3801,28 +3729,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>744:455</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="7" t="n">
+      <c r="C35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="7" t="n">
+      <c r="E35" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="F35" s="7" t="n">
+      <c r="F35" s="8" t="n">
         <v>17.1</v>
       </c>
-      <c r="G35" s="7" t="n">
-        <v>1</v>
+      <c r="G35" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -3917,28 +3845,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>746:455</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="7" t="n">
+      <c r="C39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="7" t="n">
+      <c r="E39" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F39" s="7" t="n">
+      <c r="F39" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="G39" s="7" t="n">
-        <v>1</v>
+      <c r="G39" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -3975,28 +3903,28 @@
       <c r="K40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="n">
-        <v>78</v>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>744:469</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="8" t="n">
+      <c r="A41" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>750:461</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E41" s="8" t="n">
+      <c r="E41" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F41" s="8" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G41" s="8" t="n">
-        <v>2</v>
+      <c r="F41" s="6" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
@@ -4004,28 +3932,28 @@
       <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>738:455</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="8" t="n">
+      <c r="A42" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>750:463</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E42" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="F42" s="8" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G42" s="8" t="n">
-        <v>2</v>
+      <c r="E42" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
@@ -4034,11 +3962,11 @@
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>736:457</t>
+          <t>744:469</t>
         </is>
       </c>
       <c r="C43" s="8" t="n">
@@ -4048,10 +3976,10 @@
         <v>3</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>21.8</v>
+        <v>10.5</v>
       </c>
       <c r="G43" s="8" t="n">
         <v>2</v>
@@ -4063,11 +3991,11 @@
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>740:469</t>
+          <t>738:455</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
@@ -4080,7 +4008,7 @@
         <v>24</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>14.5</v>
+        <v>21.3</v>
       </c>
       <c r="G44" s="8" t="n">
         <v>2</v>
@@ -4091,28 +4019,28 @@
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n">
-        <v>88</v>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>746:469</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="7" t="n">
+      <c r="A45" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>736:457</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="F45" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G45" s="7" t="n">
-        <v>1</v>
+      <c r="E45" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F45" s="8" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
@@ -4120,28 +4048,28 @@
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="n">
+      <c r="A46" s="6" t="n">
         <v>91</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>748:455</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="7" t="n">
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>750:459</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="F46" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>1</v>
+      <c r="E46" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
@@ -4149,28 +4077,28 @@
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="n">
+      <c r="A47" s="8" t="n">
         <v>92</v>
       </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>736:467</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="9" t="n">
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>740:469</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="F47" s="9" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G47" s="9" t="n">
-        <v>3</v>
+      <c r="E47" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G47" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
@@ -4178,28 +4106,28 @@
       <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>738:469</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="9" t="n">
+      <c r="A48" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>750:465</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E48" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="F48" s="9" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="G48" s="9" t="n">
-        <v>3</v>
+      <c r="E48" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
@@ -4207,28 +4135,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>742:453</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="8" t="n">
+      <c r="A49" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>746:469</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F49" s="8" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="G49" s="8" t="n">
-        <v>2</v>
+      <c r="F49" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -4236,28 +4164,28 @@
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="n">
-        <v>94</v>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>734:461</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="9" t="n">
+      <c r="A50" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>748:455</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F50" s="9" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <v>3</v>
+      <c r="F50" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
@@ -4265,28 +4193,28 @@
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n">
-        <v>97</v>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>744:453</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="F51" s="7" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G51" s="7" t="n">
-        <v>1</v>
+      <c r="A51" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>736:467</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G51" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
@@ -4294,28 +4222,28 @@
       <c r="K51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n">
-        <v>98</v>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>734:463</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E52" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="G52" s="9" t="n">
-        <v>3</v>
+      <c r="A52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>742:475</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
@@ -4323,28 +4251,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>742:475</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="7" t="n">
+      <c r="A53" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>740:477</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F53" s="7" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="G53" s="7" t="n">
-        <v>1</v>
+      <c r="F53" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4352,28 +4280,28 @@
       <c r="K53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>740:477</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F54" s="8" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="G54" s="8" t="n">
-        <v>2</v>
+      <c r="A54" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>744:475</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F54" s="7" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="G54" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
@@ -4381,28 +4309,28 @@
       <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>744:475</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="7" t="n">
+      <c r="A55" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>740:479</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="F55" s="7" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="G55" s="7" t="n">
-        <v>1</v>
+      <c r="F55" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G55" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -4410,28 +4338,28 @@
       <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>740:479</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="F56" s="8" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G56" s="8" t="n">
-        <v>2</v>
+      <c r="A56" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>746:477</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F56" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G56" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
@@ -4439,28 +4367,28 @@
       <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>746:477</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="7" t="n">
+      <c r="A57" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>740:475</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F57" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="G57" s="7" t="n">
-        <v>1</v>
+      <c r="F57" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -4468,28 +4396,28 @@
       <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>740:475</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="8" t="n">
+      <c r="A58" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>742:481</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F58" s="8" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="G58" s="8" t="n">
-        <v>2</v>
+      <c r="F58" s="7" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G58" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
@@ -4498,24 +4426,24 @@
     </row>
     <row r="59">
       <c r="A59" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>746:479</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>742:481</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="7" t="n">
-        <v>13</v>
-      </c>
       <c r="F59" s="7" t="n">
-        <v>17.7</v>
+        <v>13.5</v>
       </c>
       <c r="G59" s="7" t="n">
         <v>1</v>
@@ -4527,11 +4455,11 @@
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>746:479</t>
+          <t>744:481</t>
         </is>
       </c>
       <c r="C60" s="7" t="n">
@@ -4544,7 +4472,7 @@
         <v>14</v>
       </c>
       <c r="F60" s="7" t="n">
-        <v>13.5</v>
+        <v>16.3</v>
       </c>
       <c r="G60" s="7" t="n">
         <v>1</v>
@@ -4556,11 +4484,11 @@
     </row>
     <row r="61">
       <c r="A61" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>744:481</t>
+          <t>746:475</t>
         </is>
       </c>
       <c r="C61" s="7" t="n">
@@ -4570,10 +4498,10 @@
         <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>16.3</v>
+        <v>10.7</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>1</v>
@@ -4584,28 +4512,28 @@
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>746:475</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="7" t="n">
+      <c r="A62" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>740:481</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F62" s="7" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="G62" s="7" t="n">
-        <v>1</v>
+      <c r="F62" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G62" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
@@ -4613,28 +4541,28 @@
       <c r="K62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>740:481</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="F63" s="8" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="G63" s="8" t="n">
-        <v>2</v>
+      <c r="A63" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>746:481</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F63" s="7" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
@@ -4642,28 +4570,28 @@
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>746:481</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="F64" s="7" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="G64" s="7" t="n">
-        <v>1</v>
+      <c r="A64" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>742:473</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F64" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
@@ -4671,28 +4599,28 @@
       <c r="K64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>742:473</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="8" t="n">
+      <c r="A65" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>738:477</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="F65" s="8" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="G65" s="8" t="n">
-        <v>2</v>
+      <c r="F65" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
@@ -4700,28 +4628,28 @@
       <c r="K65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B66" s="9" t="inlineStr">
-        <is>
-          <t>738:477</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="F66" s="9" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G66" s="9" t="n">
-        <v>3</v>
+      <c r="A66" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>744:473</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="F66" s="8" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G66" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
@@ -4729,28 +4657,28 @@
       <c r="K66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="n">
-        <v>27</v>
-      </c>
-      <c r="B67" s="8" t="inlineStr">
-        <is>
-          <t>744:473</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" s="8" t="n">
+      <c r="A67" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>738:479</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="F67" s="8" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="G67" s="8" t="n">
-        <v>2</v>
+      <c r="F67" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G67" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
@@ -4758,28 +4686,28 @@
       <c r="K67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B68" s="9" t="inlineStr">
-        <is>
-          <t>738:479</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E68" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="F68" s="9" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G68" s="9" t="n">
-        <v>3</v>
+      <c r="A68" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>740:473</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="F68" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G68" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
@@ -4788,11 +4716,11 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>740:473</t>
+          <t>738:475</t>
         </is>
       </c>
       <c r="C69" s="8" t="n">
@@ -4805,7 +4733,7 @@
         <v>17</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>15.2</v>
+        <v>17.7</v>
       </c>
       <c r="G69" s="8" t="n">
         <v>2</v>
@@ -4816,28 +4744,28 @@
       <c r="K69" s="4" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="n">
-        <v>34</v>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>738:475</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D70" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E70" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="F70" s="8" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G70" s="8" t="n">
-        <v>2</v>
+      <c r="A70" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>748:477</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
@@ -4845,28 +4773,28 @@
       <c r="K70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="n">
-        <v>38</v>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
-        <is>
-          <t>748:477</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" s="7" t="n">
+      <c r="A71" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>742:483</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F71" s="7" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="G71" s="7" t="n">
-        <v>1</v>
+      <c r="F71" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G71" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
@@ -4874,28 +4802,28 @@
       <c r="K71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>742:483</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" s="8" t="n">
+      <c r="A72" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>746:473</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F72" s="8" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="G72" s="8" t="n">
-        <v>2</v>
+      <c r="F72" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
@@ -4904,11 +4832,11 @@
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>746:473</t>
+          <t>748:479</t>
         </is>
       </c>
       <c r="C73" s="7" t="n">
@@ -4921,7 +4849,7 @@
         <v>18</v>
       </c>
       <c r="F73" s="7" t="n">
-        <v>9.6</v>
+        <v>12.3</v>
       </c>
       <c r="G73" s="7" t="n">
         <v>1</v>
@@ -4932,28 +4860,28 @@
       <c r="K73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="n">
-        <v>44</v>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>748:479</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D74" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E74" s="7" t="n">
+      <c r="A74" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>744:483</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E74" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F74" s="7" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="G74" s="7" t="n">
-        <v>1</v>
+      <c r="F74" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H74" s="4" t="n"/>
       <c r="I74" s="4" t="n"/>
@@ -4962,11 +4890,11 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>744:483</t>
+          <t>738:481</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
@@ -4979,7 +4907,7 @@
         <v>18</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>17.9</v>
+        <v>20.7</v>
       </c>
       <c r="G75" s="8" t="n">
         <v>2</v>
@@ -4990,28 +4918,28 @@
       <c r="K75" s="4" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="9" t="n">
-        <v>48</v>
-      </c>
-      <c r="B76" s="9" t="inlineStr">
-        <is>
-          <t>738:481</t>
-        </is>
-      </c>
-      <c r="C76" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D76" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E76" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="F76" s="9" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>3</v>
+      <c r="A76" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>748:475</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G76" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
@@ -5019,28 +4947,28 @@
       <c r="K76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>748:475</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="6" t="n">
+      <c r="A77" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>740:483</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="F77" s="6" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G77" s="6" t="n">
-        <v>0</v>
+      <c r="F77" s="8" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
@@ -5049,11 +4977,11 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>740:483</t>
+          <t>748:481</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
@@ -5063,10 +4991,10 @@
         <v>2</v>
       </c>
       <c r="E78" s="8" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>20.5</v>
+        <v>14.1</v>
       </c>
       <c r="G78" s="8" t="n">
         <v>2</v>
@@ -5078,11 +5006,11 @@
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>748:481</t>
+          <t>746:483</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
@@ -5095,7 +5023,7 @@
         <v>20</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>14.1</v>
+        <v>16.8</v>
       </c>
       <c r="G79" s="8" t="n">
         <v>2</v>
@@ -5106,28 +5034,28 @@
       <c r="K79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="n">
-        <v>57</v>
-      </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>746:483</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E80" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F80" s="8" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="G80" s="8" t="n">
-        <v>2</v>
+      <c r="A80" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>748:473</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n"/>
       <c r="I80" s="4" t="n"/>
@@ -5135,28 +5063,28 @@
       <c r="K80" s="4" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="n">
-        <v>69</v>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>748:473</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D81" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E81" s="6" t="n">
+      <c r="A81" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>738:483</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F81" s="6" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="G81" s="6" t="n">
-        <v>0</v>
+      <c r="F81" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="G81" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H81" s="4" t="n"/>
       <c r="I81" s="4" t="n"/>
@@ -5164,28 +5092,28 @@
       <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="n">
-        <v>72</v>
-      </c>
-      <c r="B82" s="9" t="inlineStr">
-        <is>
-          <t>738:483</t>
-        </is>
-      </c>
-      <c r="C82" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E82" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="F82" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="G82" s="9" t="n">
-        <v>3</v>
+      <c r="A82" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>748:483</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="F82" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
@@ -5194,24 +5122,24 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>748:483</t>
+          <t>742:471</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D83" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>15.9</v>
+        <v>12.7</v>
       </c>
       <c r="G83" s="8" t="n">
         <v>2</v>
@@ -5222,28 +5150,28 @@
       <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="B84" s="8" t="inlineStr">
-        <is>
-          <t>742:471</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="8" t="n">
+      <c r="A84" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>736:477</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="8" t="n">
+      <c r="E84" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="F84" s="8" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G84" s="8" t="n">
-        <v>2</v>
+      <c r="F84" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
@@ -5251,28 +5179,28 @@
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="B85" s="9" t="inlineStr">
-        <is>
-          <t>736:477</t>
-        </is>
-      </c>
-      <c r="C85" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="9" t="n">
+      <c r="A85" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>744:471</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E85" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="F85" s="9" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G85" s="9" t="n">
-        <v>3</v>
+      <c r="E85" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F85" s="8" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G85" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
@@ -5280,28 +5208,28 @@
       <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="n">
-        <v>61</v>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
-        <is>
-          <t>744:471</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="8" t="n">
+      <c r="A86" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>736:479</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E86" s="8" t="n">
+      <c r="E86" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="F86" s="8" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="G86" s="8" t="n">
-        <v>2</v>
+      <c r="F86" s="9" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -5309,28 +5237,28 @@
       <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="9" t="n">
-        <v>64</v>
-      </c>
-      <c r="B87" s="9" t="inlineStr">
-        <is>
-          <t>736:479</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="9" t="n">
+      <c r="A87" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>740:471</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E87" s="9" t="n">
+      <c r="E87" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="F87" s="9" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G87" s="9" t="n">
-        <v>3</v>
+      <c r="F87" s="8" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H87" s="4" t="n"/>
       <c r="I87" s="4" t="n"/>
@@ -5339,11 +5267,11 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>740:471</t>
+          <t>736:475</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
@@ -5356,7 +5284,7 @@
         <v>21</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>14.7</v>
+        <v>19.6</v>
       </c>
       <c r="G88" s="8" t="n">
         <v>2</v>
@@ -5367,28 +5295,28 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="n">
-        <v>66</v>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t>736:475</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D89" s="8" t="n">
+      <c r="A89" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>746:471</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E89" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F89" s="8" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G89" s="8" t="n">
-        <v>2</v>
+      <c r="E89" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F89" s="7" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G89" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
@@ -5396,28 +5324,28 @@
       <c r="K89" s="4" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="B90" s="7" t="inlineStr">
-        <is>
-          <t>746:471</t>
-        </is>
-      </c>
-      <c r="C90" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D90" s="7" t="n">
+      <c r="A90" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>736:481</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E90" s="7" t="n">
+      <c r="E90" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F90" s="7" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G90" s="7" t="n">
-        <v>1</v>
+      <c r="F90" s="8" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="G90" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H90" s="4" t="n"/>
       <c r="I90" s="4" t="n"/>
@@ -5425,28 +5353,28 @@
       <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="9" t="n">
-        <v>76</v>
-      </c>
-      <c r="B91" s="9" t="inlineStr">
-        <is>
-          <t>736:481</t>
-        </is>
-      </c>
-      <c r="C91" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D91" s="9" t="n">
+      <c r="A91" s="7" t="n">
+        <v>78</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>750:477</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E91" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="F91" s="9" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="G91" s="9" t="n">
-        <v>3</v>
+      <c r="E91" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F91" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G91" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H91" s="4" t="n"/>
       <c r="I91" s="4" t="n"/>
@@ -5455,7 +5383,7 @@
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
@@ -5483,28 +5411,28 @@
       <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="n">
-        <v>79</v>
-      </c>
-      <c r="B93" s="8" t="inlineStr">
-        <is>
-          <t>744:485</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="8" t="n">
+      <c r="A93" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>750:479</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E93" s="8" t="n">
+      <c r="E93" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="F93" s="8" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G93" s="8" t="n">
-        <v>2</v>
+      <c r="F93" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G93" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H93" s="4" t="n"/>
       <c r="I93" s="4" t="n"/>
@@ -5513,11 +5441,11 @@
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>738:471</t>
+          <t>744:485</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
@@ -5527,10 +5455,10 @@
         <v>3</v>
       </c>
       <c r="E94" s="8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>16.7</v>
+        <v>19.6</v>
       </c>
       <c r="G94" s="8" t="n">
         <v>2</v>
@@ -5542,11 +5470,11 @@
     </row>
     <row r="95">
       <c r="A95" s="8" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>736:473</t>
+          <t>738:471</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
@@ -5559,7 +5487,7 @@
         <v>24</v>
       </c>
       <c r="F95" s="8" t="n">
-        <v>19</v>
+        <v>16.7</v>
       </c>
       <c r="G95" s="8" t="n">
         <v>2</v>
@@ -5575,7 +5503,7 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>740:485</t>
+          <t>736:473</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
@@ -5588,7 +5516,7 @@
         <v>24</v>
       </c>
       <c r="F96" s="8" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G96" s="8" t="n">
         <v>2</v>
@@ -5599,28 +5527,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="n">
-        <v>89</v>
-      </c>
-      <c r="B97" s="8" t="inlineStr">
-        <is>
-          <t>746:485</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="8" t="n">
+      <c r="A97" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>750:475</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="F97" s="8" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G97" s="8" t="n">
-        <v>2</v>
+      <c r="E97" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G97" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
@@ -5628,28 +5556,28 @@
       <c r="K97" s="4" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>748:471</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D98" s="6" t="n">
+      <c r="A98" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>740:485</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D98" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E98" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="F98" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G98" s="6" t="n">
-        <v>0</v>
+      <c r="E98" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F98" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="G98" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H98" s="4" t="n"/>
       <c r="I98" s="4" t="n"/>
@@ -5657,28 +5585,28 @@
       <c r="K98" s="4" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="9" t="n">
+      <c r="A99" s="7" t="n">
         <v>96</v>
       </c>
-      <c r="B99" s="9" t="inlineStr">
-        <is>
-          <t>736:483</t>
-        </is>
-      </c>
-      <c r="C99" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" s="9" t="n">
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>750:481</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E99" s="9" t="n">
+      <c r="E99" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F99" s="9" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G99" s="9" t="n">
-        <v>3</v>
+      <c r="F99" s="7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G99" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H99" s="4" t="n"/>
       <c r="I99" s="4" t="n"/>
@@ -5686,28 +5614,28 @@
       <c r="K99" s="4" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="B100" s="9" t="inlineStr">
-        <is>
-          <t>734:477</t>
-        </is>
-      </c>
-      <c r="C100" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E100" s="9" t="n">
+      <c r="A100" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>746:485</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E100" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="F100" s="9" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="G100" s="9" t="n">
-        <v>3</v>
+      <c r="F100" s="8" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G100" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H100" s="4" t="n"/>
       <c r="I100" s="4" t="n"/>
@@ -5715,28 +5643,28 @@
       <c r="K100" s="4" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="9" t="n">
-        <v>99</v>
-      </c>
-      <c r="B101" s="9" t="inlineStr">
-        <is>
-          <t>734:479</t>
-        </is>
-      </c>
-      <c r="C101" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D101" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E101" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="F101" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="G101" s="9" t="n">
+      <c r="A101" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>748:471</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="6" t="n">
         <v>3</v>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F101" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G101" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H101" s="4" t="n"/>
       <c r="I101" s="4" t="n"/>

</xml_diff>

<commit_message>
Map page, Mapper CSV, links
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -515,14 +515,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bear hive rollout workbook, south Fertile block. Design: alliance/bear_trap_hive.md section 16 (D2), plan: alliance/hive_rollout.md.</t>
+          <t>Bear hive rollout workbook, south block. Design history: alliance/hive_notes.md, plan: alliance/hive_plan.md.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Traps at 743:462 and 743:478, HQ stays at 755:469, 100 city slots, 20 new banners. Yellow cells are yours to fill; everything else is generated.</t>
+          <t>Traps at 743:462 and 743:478, HQ stays at 755:469, 100 city slots, 19 new banners. Yellow cells are yours to fill; everything else is generated.</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>1 Checks: does the game agree with the design? Go to each X:Y in the game, write what you see in 'Game reads', Y or N in 'OK'. Rows marked R4 need the rank.</t>
+          <t>1 Checks: does the game agree with the design? One walk through the game in the order of the rows: alliance panels (R4), HQ and banners, the block, the cluster. Write what you see in 'Game reads', Y or N in 'OK'.</t>
         </is>
       </c>
     </row>
@@ -602,17 +602,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -623,35 +624,40 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Design says</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>How to check in the game</t>
-        </is>
-      </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>How to check</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Game reads</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -663,23 +669,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>HQ tile</t>
+          <t>A. Alliance panels</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>centre 755:469, 3x3 over 754-756 / 468-470</t>
+          <t>Banner cap</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Tap the Alliance HQ, read its X:Y.</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="4" t="n"/>
+          <t>17 built, need 36</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Alliance &gt; Territory: banners built / maximum.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -687,23 +702,28 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Existing banner</t>
+          <t>A. Alliance panels</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>753:452</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Tap the banner at that spot, read its X:Y. These are the five banners nearest the block; the others are 7 apart on the same grid.</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="4" t="n"/>
+          <t>Banner cost and time</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Banner build panel: cost, build time, who can build.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -711,23 +731,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Existing banner</t>
+          <t>A. Alliance panels</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>753:459</t>
+          <t>Trap rebuild</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Tap the banner at that spot, read its X:Y. These are the five banners nearest the block; the others are 7 apart on the same grid.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="4" t="n"/>
+          <t>both traps rebuilt</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Trap panel: demolish or relocate button, cost, and whether the Pitfall level and the 2-day timer survive.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -735,23 +764,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Existing banner</t>
+          <t>A. Alliance panels</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>760:452</t>
+          <t>Alliance Bomb</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Tap the banner at that spot, read its X:Y. These are the five banners nearest the block; the others are 7 apart on the same grid.</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="4" t="n"/>
+          <t>clears vacant nodes</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Where the item is (shop, rank), its price, who may use it, cooldown.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -759,23 +797,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Existing banner</t>
+          <t>A. Alliance panels</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>760:459</t>
+          <t>Banner rule</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Tap the banner at that spot, read its X:Y. These are the five banners nearest the block; the others are 7 apart on the same grid.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="4" t="n"/>
+          <t>745:461 placeable now</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Banner placement mode, camera at 745:461: painted valid before any new banner? Its 7x7 only touches HQ territory at the edge. N = the chain must be re-solved; tell me before building anything.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -783,23 +830,28 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Existing banner</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>755:439</t>
+          <t>HQ tile</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Tap the banner at that spot, read its X:Y. These are the five banners nearest the block; the others are 7 apart on the same grid.</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="4" t="n"/>
+          <t>centre 755:469, 3x3 over 754-756 / 468-470</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Tap the Alliance HQ, read its X:Y.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -807,23 +859,28 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Resource node, quarry</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>731:451 (lower-left of its 2x2)</t>
+          <t>Existing banner</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="4" t="n"/>
+          <t>753:452</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Tap the banner, read its X:Y. The five nearest the block; the others sit 7 apart on the same grid.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -831,23 +888,28 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Resource node, woodmill</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>756:454 (lower-left of its 2x2)</t>
+          <t>Existing banner</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="4" t="n"/>
+          <t>753:459</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Tap the banner, read its X:Y. The five nearest the block; the others sit 7 apart on the same grid.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -855,23 +917,28 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>750:455 (lower-left of its 2x2)</t>
+          <t>Existing banner</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="4" t="n"/>
+          <t>760:452</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Tap the banner, read its X:Y. The five nearest the block; the others sit 7 apart on the same grid.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -879,23 +946,28 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>742:459 (lower-left of its 2x2)</t>
+          <t>Existing banner</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="4" t="n"/>
+          <t>760:459</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Tap the banner, read its X:Y. The five nearest the block; the others sit 7 apart on the same grid.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -903,23 +975,28 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>738:470 (lower-left of its 2x2)</t>
+          <t>Existing banner</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="4" t="n"/>
+          <t>755:439</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Tap the banner, read its X:Y. The five nearest the block; the others sit 7 apart on the same grid.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -927,23 +1004,28 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>B. HQ and today's banners</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>754:475 (lower-left of its 2x2)</t>
+          <t>Other banners</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="4" t="n"/>
+          <t>17 in map/banners.txt</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Any banner built since 16 Sep that is not in the list: write its X:Y in Note.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -951,23 +1033,28 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Resource node, quarry</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>736:477 (lower-left of its 2x2)</t>
+          <t>Trap 1 site</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="4" t="n"/>
+          <t>743:462, 3x3 over 742-744 / 461-463</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Is that ground empty (no city, node, water)?</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -975,23 +1062,28 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>746:479 (lower-left of its 2x2)</t>
+          <t>Trap 2 site</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="4" t="n"/>
+          <t>743:478, 3x3 over 742-744 / 477-479</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Same.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -999,23 +1091,28 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>742:485 (lower-left of its 2x2)</t>
+          <t>Node, ironmine</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="4" t="n"/>
+          <t>750:455 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1023,23 +1120,28 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>729:488 (lower-left of its 2x2)</t>
+          <t>Node, ironmine (to bomb)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="4" t="n"/>
+          <t>742:459 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1047,23 +1149,28 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Resource node, ironmine</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>748:489 (lower-left of its 2x2)</t>
+          <t>Node, ironmine (to bomb)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine (same anchor question as check 18); a missing or extra node is not.</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="4" t="n"/>
+          <t>738:470 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1071,23 +1178,28 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Lake west of the block</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>water on x 728-731, y 474-482</t>
+          <t>Node, quarry (to bomb)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Look at 730:478: water? The block's west edge (x 734) is 3 tiles from it.</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="4" t="n"/>
+          <t>736:477 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1095,23 +1207,28 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Trap 1 site</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>743:462, 3x3 over 742-744 / 461-463</t>
+          <t>Node, ironmine (to bomb)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Is that ground empty (no city, node, water)? It is Fertile Land, so foreign cities may stand there.</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="4" t="n"/>
+          <t>746:479 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1119,23 +1236,28 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Trap 2 site</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>743:478, 3x3 over 742-744 / 477-479</t>
+          <t>Node, ironmine (to bomb)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="4" t="n"/>
+          <t>742:485 (lower-left of its 2x2)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1143,23 +1265,28 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Block empty</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>x 734-749, y 453-486</t>
+          <t>Lake west of the block</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Pan over the block. Every foreign city, unknown node or odd terrain: write its X:Y in Note.</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="4" t="n"/>
+          <t>water on x 728-731, y 474-482</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Look at 730:478: water? The block's west edge (x 736) is 5 tiles from it.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1167,35 +1294,28 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2x2 anchor</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>a city's X:Y = its lower-left tile</t>
+          <t>Fertile line</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Tap your own city and one direct neighbour on the lattice. Their X:Y should differ by exactly 2. Then note which of the four tiles the readout names (walk the camera one tile at a time).</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Marsman 775:456, Lammac 777:456, Olivia1 777:458, Sting 775:458 (18 Sep 18:40); map centre on Marsman reads 776:456</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>neighbours differ by exactly 2: cities touch, 2-tile lattice confirmed; a city is named by its lower-left tile, no offset</t>
-        </is>
-      </c>
+          <t>x 749 Fertile, x 750 Plains</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Tap 749:470 and 750:470 or read the zone name. Eight seats stand on x 750 (Plains).</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1203,23 +1323,28 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Fertile line</t>
+          <t>C. The block</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>x 749 Fertile, x 750 Plains</t>
+          <t>Foreign cities</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Tap tiles 749:470 and 750:470 (or read the zone name where the map shows it). The block must be Fertile Land, the HQ must not.</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="4" t="n"/>
+          <t>none inside x 736-751, y 455-486</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Pan over the block. Every foreign city or unknown obstacle: write its X:Y in Note.</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1227,103 +1352,40 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Banner rule</t>
+          <t>D. The cluster</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>745:461 placeable before any new banner</t>
+          <t>2x2 anchor</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Banner build mode, camera at 745:461: painted valid? Its 7x7 only touches HQ territory at the edge. N = the chain must be re-solved, tell me before building anything.</t>
+          <t>a city's X:Y = its lower-left tile</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Banner cap</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>17 built, need 37</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Territory panel: banners built / maximum.</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Banner cost</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Banner build panel: cost, build time.</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Trap rebuild</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Trap panel: demolish or relocate button, cost, and whether the Pitfall level and the 2-day timer survive.</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
+          <t>Tap two cities that stand side by side; their X:Y should differ by exactly 2. DONE 18 Sep.</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Marsman 775:456, Lammac 777:456, Olivia1 777:458, Sting 775:458 (18 Sep 18:40); map centre on Marsman reads 776:456</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>neighbours differ by exactly 2: cities touch, 2-tile lattice confirmed; a city is named by its lower-left tile, no offset</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Checks 1 and 2
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -692,9 +692,21 @@
           <t>R4</t>
         </is>
       </c>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>256 built / 270 cap (18 Sep)</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>14 free, 19 needed: demolish 5 obsolete banners elsewhere before wave 2 completes, or raise the cap (alliance level)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -721,9 +733,21 @@
           <t>R4</t>
         </is>
       </c>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>stock/cost: bread 1.9M/217.8K, wood 1.0M/217.8K, stone 2.2M/145.2K, iron 2.1M/79.2K; time not shown</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>19 banners = 4.1M bread, 4.1M wood, 2.8M stone, 1.5M iron; wood covers 4 and bread 8 from stock. Garrisoning speeds the build (user).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">

</xml_diff>

<commit_message>
Three found banners, 17 new
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -733,21 +733,9 @@
           <t>R4</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>stock/cost: bread 1.9M/217.8K, wood 1.0M/217.8K, stone 2.2M/145.2K, iron 2.1M/79.2K; time not shown</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>19 banners = 4.1M bread, 4.1M wood, 2.8M stone, 1.5M iron; wood covers 4 and bread 8 from stock. Garrisoning speeds the build (user).</t>
-        </is>
-      </c>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -793,7 +781,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Alliance Bomb</t>
+          <t>Clearance Tool (the Alliance Bomb)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1159,7 +1147,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Clearance Tool (the Alliance Bomb).</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr"/>
@@ -1188,7 +1176,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Clearance Tool (the Alliance Bomb).</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr"/>
@@ -1217,7 +1205,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Clearance Tool (the Alliance Bomb).</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr"/>
@@ -1246,7 +1234,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Clearance Tool (the Alliance Bomb).</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr"/>
@@ -1275,7 +1263,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Alliance Bomb.</t>
+          <t>Find the node, read its X:Y and type. A constant offset of one tile is fine; a missing or extra node is not. This one is inside the block and gets cleared with the Clearance Tool (the Alliance Bomb).</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
@@ -1422,7 +1410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2034,110 +2022,92 @@
       <c r="J19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>744:464</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Trap 1 site 743:462; 5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="n"/>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>746:458</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>744:480</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Trap 2 site 743:478; 5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="n"/>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>754:481</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>745:461</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>3 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="n"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>746:451</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
     </row>
@@ -2152,7 +2122,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>745:477</t>
+          <t>744:480</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2161,7 +2131,7 @@
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -2170,7 +2140,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>Trap 2 site 743:478; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H23" s="4" t="n"/>
@@ -2188,7 +2158,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>752:480</t>
+          <t>739:458</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2197,7 +2167,7 @@
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -2206,7 +2176,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
+          <t>10 slots (file order)</t>
         </is>
       </c>
       <c r="H24" s="4" t="n"/>
@@ -2224,7 +2194,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>748:470</t>
+          <t>742:464</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -2233,7 +2203,7 @@
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -2242,7 +2212,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>Trap 1 site 743:462; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H25" s="4" t="n"/>
@@ -2260,7 +2230,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>750:458</t>
+          <t>745:477</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -2269,7 +2239,7 @@
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
@@ -2278,7 +2248,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H26" s="4" t="n"/>
@@ -2286,35 +2256,35 @@
       <c r="J26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>739:458</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>7 slots (file order)</t>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>752:480</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H27" s="4" t="n"/>
@@ -2322,35 +2292,35 @@
       <c r="J27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>739:474</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>7 slots (file order)</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>744:464</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H28" s="4" t="n"/>
@@ -2358,35 +2328,35 @@
       <c r="J28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n">
+      <c r="A29" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>743:470</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>9 slots (file order)</t>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>748:470</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H29" s="4" t="n"/>
@@ -2394,35 +2364,35 @@
       <c r="J29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="n">
+      <c r="A30" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>737:483</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>4 slots (file order)</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>750:483</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H30" s="4" t="n"/>
@@ -2430,35 +2400,35 @@
       <c r="J30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="n">
+      <c r="A31" s="7" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>744:487</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>8 slots (file order)</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>739:451</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H31" s="4" t="n"/>
@@ -2476,7 +2446,7 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>742:464</t>
+          <t>739:474</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -2485,7 +2455,7 @@
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
@@ -2494,7 +2464,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H32" s="4" t="n"/>
@@ -2512,7 +2482,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>750:483</t>
+          <t>743:470</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -2521,7 +2491,7 @@
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
@@ -2530,7 +2500,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>9 slots (file order)</t>
         </is>
       </c>
       <c r="H33" s="4" t="n"/>
@@ -2548,7 +2518,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>742:480</t>
+          <t>737:483</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -2557,7 +2527,7 @@
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
@@ -2566,7 +2536,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H34" s="4" t="n"/>
@@ -2584,7 +2554,7 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>744:454</t>
+          <t>744:487</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -2593,7 +2563,7 @@
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
@@ -2602,7 +2572,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>6 slots (file order)</t>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H35" s="4" t="n"/>
@@ -2610,35 +2580,35 @@
       <c r="J35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n">
+      <c r="A36" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>735:465</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>7 slots (file order)</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>742:480</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H36" s="4" t="n"/>
@@ -2646,35 +2616,35 @@
       <c r="J36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="n">
+      <c r="A37" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>735:476</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>4 slots (file order)</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>736:469</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>2 slots (file order)</t>
         </is>
       </c>
       <c r="H37" s="4" t="n"/>
@@ -2682,35 +2652,35 @@
       <c r="J37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n">
+      <c r="A38" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>736:469</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>1 slots (file order)</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>735:463</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>6 slots (file order)</t>
         </is>
       </c>
       <c r="H38" s="4" t="n"/>
@@ -2718,33 +2688,35 @@
       <c r="J38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="n">
+      <c r="A39" s="9" t="n">
         <v>37</v>
       </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr"/>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>banner 744:464 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G39" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>735:476</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>wave 3</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>wave 2 complete</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H39" s="4" t="n"/>
@@ -2757,12 +2729,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>743:478</t>
+          <t>743:462</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
@@ -2773,7 +2745,7 @@
       <c r="E40" s="10" t="inlineStr"/>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>banner 744:480 (wave 1); the old trap's last firing</t>
+          <t>banner 742:464 (wave 1); the old trap's last firing</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
@@ -2784,6 +2756,40 @@
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
       <c r="J40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr"/>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>banner 744:480 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2899,28 +2905,28 @@
       <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>740:461</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="8" t="n">
+      <c r="C3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="7" t="n">
         <v>16.3</v>
       </c>
-      <c r="G3" s="8" t="n">
-        <v>2</v>
+      <c r="G3" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
@@ -2928,28 +2934,28 @@
       <c r="K3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>744:459</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7" t="n">
+      <c r="C4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="6" t="n">
         <v>14.2</v>
       </c>
-      <c r="G4" s="7" t="n">
-        <v>1</v>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
@@ -2957,28 +2963,28 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>740:463</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8" t="n">
+      <c r="C5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="7" t="n">
         <v>15.5</v>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>2</v>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
@@ -3044,28 +3050,28 @@
       <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>740:459</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="8" t="n">
+      <c r="C8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="7" t="n">
         <v>17.3</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>2</v>
+      <c r="G8" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
@@ -3131,28 +3137,28 @@
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>746:459</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="7" t="n">
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="6" t="n">
         <v>12.7</v>
       </c>
-      <c r="G11" s="7" t="n">
-        <v>1</v>
+      <c r="G11" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
@@ -3160,28 +3166,28 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>740:465</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="8" t="n">
+      <c r="C12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="7" t="n">
         <v>14.9</v>
       </c>
-      <c r="G12" s="8" t="n">
-        <v>2</v>
+      <c r="G12" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
@@ -3218,28 +3224,28 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>742:457</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="8" t="n">
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="G14" s="8" t="n">
-        <v>2</v>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
@@ -3247,28 +3253,28 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n">
+      <c r="A15" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>738:461</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="9" t="n">
+      <c r="C15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="8" t="n">
         <v>18.1</v>
       </c>
-      <c r="G15" s="9" t="n">
-        <v>3</v>
+      <c r="G15" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -3276,28 +3282,28 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>744:457</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="8" t="n">
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="6" t="n">
         <v>15.6</v>
       </c>
-      <c r="G16" s="8" t="n">
-        <v>2</v>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -3305,28 +3311,28 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n">
+      <c r="A17" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>738:463</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="9" t="n">
+      <c r="C17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="8" t="n">
         <v>17.4</v>
       </c>
-      <c r="G17" s="9" t="n">
-        <v>3</v>
+      <c r="G17" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -3334,28 +3340,28 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>740:457</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="n">
+      <c r="C18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="7" t="n">
         <v>18.5</v>
       </c>
-      <c r="G18" s="8" t="n">
-        <v>2</v>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
@@ -3363,28 +3369,28 @@
       <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>738:459</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="8" t="n">
+      <c r="C19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="G19" s="8" t="n">
-        <v>2</v>
+      <c r="G19" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
@@ -3392,28 +3398,28 @@
       <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>748:461</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="7" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="6" t="n">
         <v>9.9</v>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
+      <c r="G20" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -3513,7 +3519,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>746:457</t>
+          <t>738:465</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
@@ -3526,7 +3532,7 @@
         <v>18</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>14.3</v>
+        <v>16.9</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>2</v>
@@ -3537,28 +3543,28 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>738:465</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>3</v>
+      <c r="A25" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>748:459</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -3566,28 +3572,28 @@
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>748:459</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="7" t="n">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>740:467</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="F26" s="7" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
+      <c r="F26" s="8" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
@@ -3595,28 +3601,28 @@
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>740:467</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="F27" s="8" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G27" s="8" t="n">
-        <v>2</v>
+      <c r="A27" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>748:465</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -3624,28 +3630,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="7" t="n">
         <v>53</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>748:465</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="6" t="n">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>746:467</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>0</v>
+      <c r="F28" s="7" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -3653,28 +3659,28 @@
       <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n">
-        <v>54</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>746:467</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F29" s="7" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="G29" s="7" t="n">
-        <v>1</v>
+      <c r="A29" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>748:457</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
@@ -3682,28 +3688,28 @@
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>748:457</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="7" t="n">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>738:467</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F30" s="7" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>1</v>
+      <c r="F30" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
@@ -3711,28 +3717,28 @@
       <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="n">
-        <v>71</v>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>738:467</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>3</v>
+      <c r="A31" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>748:467</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
@@ -3740,28 +3746,28 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>84</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>748:467</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>0</v>
+      <c r="A32" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>742:455</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -3774,7 +3780,7 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>742:455</t>
+          <t>736:461</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
@@ -3787,7 +3793,7 @@
         <v>20</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>18.4</v>
+        <v>20</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>2</v>
@@ -3798,28 +3804,28 @@
       <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>736:461</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="9" t="n">
+      <c r="A34" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>744:455</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E34" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <v>3</v>
+      <c r="E34" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
@@ -3832,7 +3838,7 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>744:455</t>
+          <t>736:463</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
@@ -3845,7 +3851,7 @@
         <v>21</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>17.1</v>
+        <v>19.3</v>
       </c>
       <c r="G35" s="8" t="n">
         <v>2</v>
@@ -3856,28 +3862,28 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n">
-        <v>63</v>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>736:463</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="9" t="n">
+      <c r="A36" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>740:455</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="9" t="n">
+      <c r="E36" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F36" s="9" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G36" s="9" t="n">
-        <v>3</v>
+      <c r="F36" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
@@ -3885,28 +3891,28 @@
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n">
+      <c r="A37" s="7" t="n">
         <v>67</v>
       </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>740:455</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="8" t="n">
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>736:459</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="8" t="n">
+      <c r="E37" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F37" s="8" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G37" s="8" t="n">
-        <v>2</v>
+      <c r="F37" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
@@ -3914,28 +3920,28 @@
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="n">
-        <v>68</v>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>736:459</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="8" t="n">
+      <c r="A38" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>746:455</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F38" s="8" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="G38" s="8" t="n">
-        <v>2</v>
+      <c r="E38" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
@@ -3948,7 +3954,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>746:455</t>
+          <t>736:465</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
@@ -3961,7 +3967,7 @@
         <v>22</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>16</v>
+        <v>18.8</v>
       </c>
       <c r="G39" s="8" t="n">
         <v>2</v>
@@ -3972,28 +3978,28 @@
       <c r="K39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="n">
-        <v>75</v>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>736:465</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="9" t="n">
+      <c r="A40" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>750:461</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E40" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <v>3</v>
+      <c r="E40" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4" t="n"/>
@@ -4002,11 +4008,11 @@
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>750:461</t>
+          <t>750:463</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
@@ -4019,7 +4025,7 @@
         <v>23</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>8.699999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="G41" s="6" t="n">
         <v>0</v>
@@ -4030,28 +4036,28 @@
       <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>750:463</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="6" t="n">
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>744:469</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E42" s="6" t="n">
+      <c r="E42" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="F42" s="6" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>0</v>
+      <c r="F42" s="8" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G42" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
@@ -4059,28 +4065,28 @@
       <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="n">
-        <v>81</v>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>744:469</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="8" t="n">
+      <c r="A43" s="7" t="n">
+        <v>87</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>738:455</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="F43" s="8" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G43" s="8" t="n">
-        <v>2</v>
+      <c r="E43" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
@@ -4088,28 +4094,28 @@
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="n">
+      <c r="A44" s="7" t="n">
         <v>88</v>
       </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>738:455</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="8" t="n">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>736:457</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="8" t="n">
+      <c r="E44" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="F44" s="8" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G44" s="8" t="n">
-        <v>2</v>
+      <c r="F44" s="7" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
@@ -4117,28 +4123,28 @@
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="n">
-        <v>89</v>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>736:457</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="8" t="n">
+      <c r="A45" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>750:459</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="E45" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="F45" s="8" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="G45" s="8" t="n">
-        <v>2</v>
+      <c r="F45" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
@@ -4146,28 +4152,28 @@
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="8" t="n">
         <v>91</v>
       </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>750:459</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="6" t="n">
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>740:469</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="6" t="n">
+      <c r="E46" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="F46" s="6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G46" s="6" t="n">
-        <v>0</v>
+      <c r="F46" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
@@ -4175,28 +4181,28 @@
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>740:469</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="8" t="n">
+      <c r="A47" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>750:465</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="F47" s="8" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G47" s="8" t="n">
-        <v>2</v>
+      <c r="E47" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
@@ -4204,28 +4210,28 @@
       <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="7" t="n">
         <v>94</v>
       </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>750:465</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="6" t="n">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>746:469</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E48" s="6" t="n">
+      <c r="E48" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F48" s="6" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>0</v>
+      <c r="F48" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
@@ -4233,28 +4239,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
-        <v>95</v>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>746:469</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="7" t="n">
+      <c r="A49" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>748:455</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="7" t="n">
+      <c r="E49" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F49" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G49" s="7" t="n">
-        <v>1</v>
+      <c r="F49" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -4262,28 +4268,28 @@
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>748:455</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="7" t="n">
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>736:467</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E50" s="7" t="n">
+      <c r="E50" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="F50" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="G50" s="7" t="n">
-        <v>1</v>
+      <c r="F50" s="8" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
@@ -4291,28 +4297,28 @@
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="n">
+      <c r="A51" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>736:467</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E51" s="9" t="n">
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>742:453</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F51" s="9" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <v>3</v>
+      <c r="F51" s="7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
@@ -4959,7 +4965,7 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
@@ -4988,7 +4994,7 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
@@ -5017,7 +5023,7 @@
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
@@ -5046,7 +5052,7 @@
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
@@ -5074,28 +5080,28 @@
       <c r="K77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="A78" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
         <is>
           <t>748:481</t>
         </is>
       </c>
-      <c r="C78" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D78" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E78" s="8" t="n">
+      <c r="C78" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F78" s="7" t="n">
         <v>14.1</v>
       </c>
-      <c r="G78" s="8" t="n">
-        <v>2</v>
+      <c r="G78" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
@@ -5104,7 +5110,7 @@
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
@@ -5133,7 +5139,7 @@
     </row>
     <row r="80">
       <c r="A80" s="6" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
@@ -5162,7 +5168,7 @@
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
@@ -5190,28 +5196,28 @@
       <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="A82" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>748:483</t>
         </is>
       </c>
-      <c r="C82" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E82" s="8" t="n">
+      <c r="C82" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="F82" s="8" t="n">
+      <c r="F82" s="7" t="n">
         <v>15.9</v>
       </c>
-      <c r="G82" s="8" t="n">
-        <v>2</v>
+      <c r="G82" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
@@ -5220,7 +5226,7 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
@@ -5249,7 +5255,7 @@
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
@@ -5278,7 +5284,7 @@
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
@@ -5307,7 +5313,7 @@
     </row>
     <row r="86">
       <c r="A86" s="9" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B86" s="9" t="inlineStr">
         <is>
@@ -5336,7 +5342,7 @@
     </row>
     <row r="87">
       <c r="A87" s="8" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
@@ -5365,7 +5371,7 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
@@ -5394,7 +5400,7 @@
     </row>
     <row r="89">
       <c r="A89" s="7" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
@@ -5423,7 +5429,7 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
@@ -5452,7 +5458,7 @@
     </row>
     <row r="91">
       <c r="A91" s="7" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
@@ -5481,7 +5487,7 @@
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
@@ -5510,7 +5516,7 @@
     </row>
     <row r="93">
       <c r="A93" s="7" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
@@ -5539,7 +5545,7 @@
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
@@ -5568,7 +5574,7 @@
     </row>
     <row r="95">
       <c r="A95" s="8" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
@@ -5597,7 +5603,7 @@
     </row>
     <row r="96">
       <c r="A96" s="8" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
@@ -5626,7 +5632,7 @@
     </row>
     <row r="97">
       <c r="A97" s="6" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
@@ -5655,7 +5661,7 @@
     </row>
     <row r="98">
       <c r="A98" s="8" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
@@ -5684,7 +5690,7 @@
     </row>
     <row r="99">
       <c r="A99" s="7" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
@@ -5713,7 +5719,7 @@
     </row>
     <row r="100">
       <c r="A100" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
@@ -5742,7 +5748,7 @@
     </row>
     <row r="101">
       <c r="A101" s="6" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ring 4 seats moved into ring 3
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -2720,7 +2720,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>10 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H42" s="4" t="n"/>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>12 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H49" s="4" t="n"/>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>10 slots (file order)</t>
+          <t>9 slots (file order)</t>
         </is>
       </c>
       <c r="H50" s="4" t="n"/>
@@ -4539,7 +4539,7 @@
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
@@ -4567,28 +4567,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
-        <v>97</v>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>744:453</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G49" s="6" t="n">
-        <v>0</v>
+      <c r="A49" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>736:455</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F49" s="7" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -4596,28 +4596,28 @@
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>734:465</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="8" t="n">
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>750:467</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="F50" s="8" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="G50" s="8" t="n">
-        <v>2</v>
+      <c r="F50" s="6" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
@@ -6047,7 +6047,7 @@
     </row>
     <row r="100">
       <c r="A100" s="6" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
@@ -6076,24 +6076,24 @@
     </row>
     <row r="101">
       <c r="A101" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>734:479</t>
+          <t>736:471</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D101" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F101" s="8" t="n">
-        <v>23</v>
+        <v>18.7</v>
       </c>
       <c r="G101" s="8" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
HQ territory corrected (starts x 749, y 463): 14 banners, 3 built; banner map, map page, workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E8D3F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F5C6B8"/>
       </patternFill>
     </fill>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,6 +136,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -514,7 +522,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Traps at 743:462 and 743:478, HQ stays at 755:469, 100 city slots, 19 new banners. Yellow cells are yours to fill; everything else is generated.</t>
+          <t>Traps at 743:462 and 743:478, HQ stays at 755:469, 100 city slots, 14 new banners. Yellow cells are yours to fill; everything else is generated.</t>
         </is>
       </c>
     </row>
@@ -792,8 +800,16 @@
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>count and radius unknown; not to be asked again (user 18 Sep). Will show when the tool is used.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -811,12 +827,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>745:461 placeable now</t>
+          <t>edge contact is enough</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Banner placement mode, camera at 745:461: painted valid before any new banner? Its 7x7 only touches HQ territory at the edge. N = the chain must be re-solved; tell me before building anything.</t>
+          <t>DONE 19 Sep: 745:477 was built with its 7x7 only abutting the HQ territory edge (x 748 | 749). A new banner may touch existing territory edge to edge.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -844,12 +860,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>centre 755:469, 3x3 over 754-756 / 468-470</t>
+          <t>755:469 = lower-left tile, 3x3 over 755-757 / 469-471</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Tap the Alliance HQ, read its X:Y.</t>
+          <t>DONE 19 Sep: territory ends at x 749 (gap at 748:470 to a banner reaching 747). The game names a 3x3 by its lower-left tile, like a city.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
@@ -1414,7 +1430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1504,7 +1520,7 @@
       <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>15x15 territory x 748-762, y 462-476; six slots stand on it today</t>
+          <t>15x15 territory x 749-763, y 463-477 (game-verified 19 Sep); 755:469 is its lower-left tile</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -2666,7 +2682,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>744:480</t>
+          <t>745:477</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -2684,11 +2700,19 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Trap 2 site 743:478; 5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
+          <t>Trap 2 site 743:478; 6 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J41" s="4" t="n"/>
     </row>
     <row r="42">
@@ -2711,7 +2735,7 @@
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -2738,7 +2762,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>745:477</t>
+          <t>752:480</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -2747,7 +2771,7 @@
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
@@ -2756,7 +2780,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H43" s="4" t="n"/>
@@ -2774,7 +2798,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>752:480</t>
+          <t>744:464</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2783,7 +2807,7 @@
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -2792,7 +2816,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
+          <t>Trap 1 site 743:462; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H44" s="4" t="n"/>
@@ -2810,7 +2834,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>744:464</t>
+          <t>750:483</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -2819,7 +2843,7 @@
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
@@ -2828,7 +2852,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Trap 1 site 743:462; 5 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H45" s="4" t="n"/>
@@ -2846,7 +2870,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>750:483</t>
+          <t>745:464</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2855,7 +2879,7 @@
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -2882,7 +2906,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>744:470</t>
+          <t>745:470</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2891,7 +2915,7 @@
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2900,7 +2924,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>10 slots (file order)</t>
+          <t>3 slots (file order)</t>
         </is>
       </c>
       <c r="H47" s="4" t="n"/>
@@ -2908,35 +2932,35 @@
       <c r="J47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="n">
+      <c r="A48" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>739:474</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>8 slots (file order)</t>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>752:459</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
@@ -2954,7 +2978,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>737:465</t>
+          <t>744:480</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -2963,7 +2987,7 @@
         </is>
       </c>
       <c r="E49" s="8" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
@@ -2972,11 +2996,19 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>11 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
+          <t>3 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J49" s="4" t="n"/>
     </row>
     <row r="50">
@@ -2990,7 +3022,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>737:481</t>
+          <t>743:487</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -2999,7 +3031,7 @@
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
@@ -3008,11 +3040,19 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>9 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
+          <t>5 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J50" s="4" t="n"/>
     </row>
     <row r="51">
@@ -3026,7 +3066,7 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>743:487</t>
+          <t>744:470</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -3035,7 +3075,7 @@
         </is>
       </c>
       <c r="E51" s="8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
@@ -3044,7 +3084,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>8 slots (file order)</t>
+          <t>10 slots (file order)</t>
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
@@ -3052,33 +3092,35 @@
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n">
+      <c r="A52" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr"/>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>banner 744:464 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>739:474</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
@@ -3086,38 +3128,144 @@
       <c r="J52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
+      <c r="A53" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="inlineStr"/>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>banner 744:480 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>737:465</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
       <c r="J53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>737:481</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>wave 3</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>wave 2 complete</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>10 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
+      <c r="J54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr"/>
+      <c r="F55" s="10" t="inlineStr">
+        <is>
+          <t>banner 744:464 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G55" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="inlineStr"/>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>banner 745:477 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
+      <c r="J56" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3726,28 +3874,28 @@
       <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="8" t="n">
         <v>37</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>742:467</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="7" t="n">
+      <c r="C20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="8" t="n">
         <v>12.6</v>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
+      <c r="G20" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -3755,28 +3903,28 @@
       <c r="K20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="7" t="n">
         <v>39</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>748:461</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="6" t="n">
+      <c r="C21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F21" s="7" t="n">
         <v>9.9</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>0</v>
+      <c r="G21" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
@@ -3813,28 +3961,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>744:467</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="7" t="n">
+      <c r="C23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="7" t="n">
+      <c r="F23" s="8" t="n">
         <v>10.6</v>
       </c>
-      <c r="G23" s="7" t="n">
-        <v>1</v>
+      <c r="G23" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -3842,28 +3990,28 @@
       <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>748:463</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="6" t="n">
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F24" s="7" t="n">
         <v>8.5</v>
       </c>
-      <c r="G24" s="6" t="n">
-        <v>0</v>
+      <c r="G24" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -3929,28 +4077,28 @@
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>746:467</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="7" t="n">
+      <c r="C27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F27" s="7" t="n">
+      <c r="F27" s="8" t="n">
         <v>8.6</v>
       </c>
-      <c r="G27" s="7" t="n">
-        <v>1</v>
+      <c r="G27" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -3958,28 +4106,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="7" t="n">
         <v>58</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>748:465</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="6" t="n">
+      <c r="C28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="F28" s="7" t="n">
         <v>7.4</v>
       </c>
-      <c r="G28" s="6" t="n">
-        <v>0</v>
+      <c r="G28" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -4045,28 +4193,28 @@
       <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>748:467</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="6" t="n">
+      <c r="C31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F31" s="7" t="n">
         <v>6.7</v>
       </c>
-      <c r="G31" s="6" t="n">
-        <v>0</v>
+      <c r="G31" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
@@ -4422,28 +4570,28 @@
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>746:469</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="7" t="n">
+      <c r="C44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="7" t="n">
+      <c r="E44" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="F44" s="7" t="n">
+      <c r="F44" s="8" t="n">
         <v>8.5</v>
       </c>
-      <c r="G44" s="7" t="n">
-        <v>1</v>
+      <c r="G44" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
@@ -4625,28 +4773,28 @@
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="A51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>740:477</t>
         </is>
       </c>
-      <c r="C51" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="8" t="n">
+      <c r="C51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="9" t="n">
         <v>16.8</v>
       </c>
-      <c r="G51" s="8" t="n">
-        <v>2</v>
+      <c r="G51" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
@@ -4683,28 +4831,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="n">
+      <c r="A53" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>740:479</t>
         </is>
       </c>
-      <c r="C53" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="8" t="n">
+      <c r="C53" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F53" s="9" t="n">
         <v>17.9</v>
       </c>
-      <c r="G53" s="8" t="n">
-        <v>2</v>
+      <c r="G53" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4770,28 +4918,28 @@
       <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n">
+      <c r="A56" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>742:481</t>
         </is>
       </c>
-      <c r="C56" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="7" t="n">
+      <c r="C56" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F56" s="7" t="n">
+      <c r="F56" s="8" t="n">
         <v>17.7</v>
       </c>
-      <c r="G56" s="7" t="n">
-        <v>1</v>
+      <c r="G56" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
@@ -4828,28 +4976,28 @@
       <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="n">
+      <c r="A58" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>744:481</t>
         </is>
       </c>
-      <c r="C58" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="7" t="n">
+      <c r="C58" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="F58" s="7" t="n">
+      <c r="F58" s="8" t="n">
         <v>16.3</v>
       </c>
-      <c r="G58" s="7" t="n">
-        <v>1</v>
+      <c r="G58" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
@@ -4886,28 +5034,28 @@
       <c r="K59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n">
+      <c r="A60" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t>740:481</t>
         </is>
       </c>
-      <c r="C60" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="8" t="n">
+      <c r="C60" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="F60" s="8" t="n">
+      <c r="F60" s="9" t="n">
         <v>19.1</v>
       </c>
-      <c r="G60" s="8" t="n">
-        <v>2</v>
+      <c r="G60" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
@@ -4944,28 +5092,28 @@
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="n">
+      <c r="A62" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>746:481</t>
         </is>
       </c>
-      <c r="C62" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="7" t="n">
+      <c r="C62" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F62" s="7" t="n">
+      <c r="F62" s="8" t="n">
         <v>15.1</v>
       </c>
-      <c r="G62" s="7" t="n">
-        <v>1</v>
+      <c r="G62" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
@@ -4973,28 +5121,28 @@
       <c r="K62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="n">
+      <c r="A63" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>738:477</t>
         </is>
       </c>
-      <c r="C63" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="8" t="n">
+      <c r="C63" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="F63" s="9" t="n">
         <v>18.6</v>
       </c>
-      <c r="G63" s="8" t="n">
-        <v>2</v>
+      <c r="G63" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
@@ -5002,28 +5150,28 @@
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="n">
+      <c r="A64" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>742:473</t>
         </is>
       </c>
-      <c r="C64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E64" s="7" t="n">
+      <c r="C64" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F64" s="7" t="n">
+      <c r="F64" s="8" t="n">
         <v>13.3</v>
       </c>
-      <c r="G64" s="7" t="n">
-        <v>1</v>
+      <c r="G64" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
@@ -5031,28 +5179,28 @@
       <c r="K64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="n">
+      <c r="A65" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>738:479</t>
         </is>
       </c>
-      <c r="C65" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="8" t="n">
+      <c r="C65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="F65" s="8" t="n">
+      <c r="F65" s="9" t="n">
         <v>19.6</v>
       </c>
-      <c r="G65" s="8" t="n">
-        <v>2</v>
+      <c r="G65" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
@@ -5060,28 +5208,28 @@
       <c r="K65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="n">
+      <c r="A66" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B66" s="7" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>744:473</t>
         </is>
       </c>
-      <c r="C66" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" s="7" t="n">
+      <c r="C66" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F66" s="7" t="n">
+      <c r="F66" s="8" t="n">
         <v>11.4</v>
       </c>
-      <c r="G66" s="7" t="n">
-        <v>1</v>
+      <c r="G66" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
@@ -5205,28 +5353,28 @@
       <c r="K70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="n">
+      <c r="A71" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>738:481</t>
         </is>
       </c>
-      <c r="C71" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" s="8" t="n">
+      <c r="C71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="F71" s="8" t="n">
+      <c r="F71" s="9" t="n">
         <v>20.7</v>
       </c>
-      <c r="G71" s="8" t="n">
-        <v>2</v>
+      <c r="G71" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
@@ -5263,28 +5411,28 @@
       <c r="K72" s="4" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="n">
+      <c r="A73" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="B73" s="8" t="inlineStr">
         <is>
           <t>746:473</t>
         </is>
       </c>
-      <c r="C73" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="7" t="n">
+      <c r="C73" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="F73" s="7" t="n">
+      <c r="F73" s="8" t="n">
         <v>9.6</v>
       </c>
-      <c r="G73" s="7" t="n">
-        <v>1</v>
+      <c r="G73" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="n"/>
@@ -5321,28 +5469,28 @@
       <c r="K74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="n">
+      <c r="A75" s="9" t="n">
         <v>49</v>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="9" t="inlineStr">
         <is>
           <t>740:483</t>
         </is>
       </c>
-      <c r="C75" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D75" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" s="8" t="n">
+      <c r="C75" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="F75" s="8" t="n">
+      <c r="F75" s="9" t="n">
         <v>20.5</v>
       </c>
-      <c r="G75" s="8" t="n">
-        <v>2</v>
+      <c r="G75" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
@@ -5350,28 +5498,28 @@
       <c r="K75" s="4" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="n">
+      <c r="A76" s="7" t="n">
         <v>51</v>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B76" s="7" t="inlineStr">
         <is>
           <t>748:475</t>
         </is>
       </c>
-      <c r="C76" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D76" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E76" s="6" t="n">
+      <c r="C76" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="F76" s="6" t="n">
+      <c r="F76" s="7" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="G76" s="6" t="n">
-        <v>0</v>
+      <c r="G76" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
@@ -5379,28 +5527,28 @@
       <c r="K76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="n">
+      <c r="A77" s="7" t="n">
         <v>57</v>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>746:483</t>
         </is>
       </c>
-      <c r="C77" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="8" t="n">
+      <c r="C77" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F77" s="8" t="n">
+      <c r="F77" s="7" t="n">
         <v>16.8</v>
       </c>
-      <c r="G77" s="8" t="n">
-        <v>2</v>
+      <c r="G77" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
@@ -5437,28 +5585,28 @@
       <c r="K78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="n">
+      <c r="A79" s="9" t="n">
         <v>69</v>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B79" s="9" t="inlineStr">
         <is>
           <t>738:483</t>
         </is>
       </c>
-      <c r="C79" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D79" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" s="8" t="n">
+      <c r="C79" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="F79" s="8" t="n">
+      <c r="F79" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="G79" s="8" t="n">
-        <v>2</v>
+      <c r="G79" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
@@ -5466,28 +5614,28 @@
       <c r="K79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="n">
+      <c r="A80" s="7" t="n">
         <v>71</v>
       </c>
-      <c r="B80" s="6" t="inlineStr">
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>748:473</t>
         </is>
       </c>
-      <c r="C80" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E80" s="6" t="n">
+      <c r="C80" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E80" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F80" s="6" t="n">
+      <c r="F80" s="7" t="n">
         <v>7.9</v>
       </c>
-      <c r="G80" s="6" t="n">
-        <v>0</v>
+      <c r="G80" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H80" s="4" t="n"/>
       <c r="I80" s="4" t="n"/>
@@ -5524,28 +5672,28 @@
       <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="n">
+      <c r="A82" s="9" t="n">
         <v>53</v>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>736:477</t>
         </is>
       </c>
-      <c r="C82" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="8" t="n">
+      <c r="C82" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E82" s="8" t="n">
+      <c r="E82" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="F82" s="8" t="n">
+      <c r="F82" s="9" t="n">
         <v>20.4</v>
       </c>
-      <c r="G82" s="8" t="n">
-        <v>2</v>
+      <c r="G82" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
@@ -5553,28 +5701,28 @@
       <c r="K82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="n">
+      <c r="A83" s="8" t="n">
         <v>55</v>
       </c>
-      <c r="B83" s="7" t="inlineStr">
+      <c r="B83" s="8" t="inlineStr">
         <is>
           <t>742:471</t>
         </is>
       </c>
-      <c r="C83" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D83" s="7" t="n">
+      <c r="C83" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E83" s="7" t="n">
+      <c r="E83" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F83" s="7" t="n">
+      <c r="F83" s="8" t="n">
         <v>12.7</v>
       </c>
-      <c r="G83" s="7" t="n">
-        <v>1</v>
+      <c r="G83" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H83" s="4" t="n"/>
       <c r="I83" s="4" t="n"/>
@@ -5582,28 +5730,28 @@
       <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="n">
+      <c r="A84" s="9" t="n">
         <v>61</v>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>736:479</t>
         </is>
       </c>
-      <c r="C84" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="8" t="n">
+      <c r="C84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="8" t="n">
+      <c r="E84" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="F84" s="8" t="n">
+      <c r="F84" s="9" t="n">
         <v>21.3</v>
       </c>
-      <c r="G84" s="8" t="n">
-        <v>2</v>
+      <c r="G84" s="9" t="n">
+        <v>3</v>
       </c>
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
@@ -5611,28 +5759,28 @@
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="n">
+      <c r="A85" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="B85" s="8" t="inlineStr">
         <is>
           <t>744:471</t>
         </is>
       </c>
-      <c r="C85" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="7" t="n">
+      <c r="C85" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E85" s="7" t="n">
+      <c r="E85" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="F85" s="7" t="n">
+      <c r="F85" s="8" t="n">
         <v>10.8</v>
       </c>
-      <c r="G85" s="7" t="n">
-        <v>1</v>
+      <c r="G85" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
@@ -5698,28 +5846,28 @@
       <c r="K87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="7" t="n">
+      <c r="A88" s="8" t="n">
         <v>73</v>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B88" s="8" t="inlineStr">
         <is>
           <t>746:471</t>
         </is>
       </c>
-      <c r="C88" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="7" t="n">
+      <c r="C88" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E88" s="7" t="n">
+      <c r="E88" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="F88" s="7" t="n">
+      <c r="F88" s="8" t="n">
         <v>8.9</v>
       </c>
-      <c r="G88" s="7" t="n">
-        <v>1</v>
+      <c r="G88" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H88" s="4" t="n"/>
       <c r="I88" s="4" t="n"/>
@@ -5959,28 +6107,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="n">
+      <c r="A97" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>746:485</t>
         </is>
       </c>
-      <c r="C97" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="8" t="n">
+      <c r="C97" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="8" t="n">
+      <c r="E97" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F97" s="8" t="n">
+      <c r="F97" s="7" t="n">
         <v>18.6</v>
       </c>
-      <c r="G97" s="8" t="n">
-        <v>2</v>
+      <c r="G97" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
@@ -6017,28 +6165,28 @@
       <c r="K98" s="4" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="n">
+      <c r="A99" s="7" t="n">
         <v>95</v>
       </c>
-      <c r="B99" s="6" t="inlineStr">
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>748:471</t>
         </is>
       </c>
-      <c r="C99" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" s="6" t="n">
+      <c r="C99" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E99" s="6" t="n">
+      <c r="E99" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="F99" s="6" t="n">
+      <c r="F99" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="G99" s="6" t="n">
-        <v>0</v>
+      <c r="G99" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H99" s="4" t="n"/>
       <c r="I99" s="4" t="n"/>

</xml_diff>

<commit_message>
Redesign with the HQ territory at x 749-763, y 463-477: 7 new banners (3 built stay), seats regenerated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -74,11 +74,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D3F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F5C6B8"/>
       </patternFill>
     </fill>
@@ -109,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -136,9 +131,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1430,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2672,35 +2664,31 @@
       <c r="J40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>745:477</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>Trap 2 site 743:478; 6 slots (file order)</t>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2716,75 +2704,83 @@
       <c r="J41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n">
+      <c r="A42" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>739:458</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>744:480</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>752:480</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>743:487</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="6" t="inlineStr"/>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J43" s="4" t="n"/>
     </row>
     <row r="44">
@@ -2798,7 +2794,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>744:464</t>
+          <t>739:457</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2807,7 +2803,7 @@
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -2816,7 +2812,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Trap 1 site 743:462; 5 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H44" s="4" t="n"/>
@@ -2834,7 +2830,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>750:483</t>
+          <t>744:464</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -2843,7 +2839,7 @@
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
@@ -2852,7 +2848,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>4 slots (file order)</t>
+          <t>Trap 1 site 743:462; 5 slots (file order)</t>
         </is>
       </c>
       <c r="H45" s="4" t="n"/>
@@ -2870,7 +2866,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>745:464</t>
+          <t>745:470</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2879,7 +2875,7 @@
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -2888,7 +2884,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>2 slots (file order)</t>
+          <t>15 slots (file order)</t>
         </is>
       </c>
       <c r="H46" s="4" t="n"/>
@@ -2906,7 +2902,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>745:470</t>
+          <t>738:473</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2915,7 +2911,7 @@
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2924,7 +2920,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>3 slots (file order)</t>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H47" s="4" t="n"/>
@@ -2942,7 +2938,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>752:459</t>
+          <t>737:480</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2951,7 +2947,7 @@
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -2960,7 +2956,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>1 slots (file order)</t>
+          <t>12 slots (file order)</t>
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
@@ -2968,47 +2964,39 @@
       <c r="J48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="n">
+      <c r="A49" s="7" t="n">
         <v>47</v>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>744:480</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G49" s="8" t="inlineStr">
-        <is>
-          <t>3 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>750:481</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>7 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
       <c r="J49" s="4" t="n"/>
     </row>
     <row r="50">
@@ -3022,7 +3010,7 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>743:487</t>
+          <t>737:463</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -3031,7 +3019,7 @@
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
@@ -3040,51 +3028,41 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
+          <t>11 slots (file order)</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
       <c r="J50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="n">
+      <c r="A51" s="9" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>744:470</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G51" s="8" t="inlineStr">
-        <is>
-          <t>10 slots (file order)</t>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>banner 744:464 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
@@ -3092,180 +3070,38 @@
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>739:474</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="inlineStr">
-        <is>
-          <t>8 slots (file order)</t>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr"/>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>banner 745:477 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
       <c r="J52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>737:465</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G53" s="8" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>737:481</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>wave 3</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>wave 2 complete</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
-        <is>
-          <t>10 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr"/>
-      <c r="F55" s="10" t="inlineStr">
-        <is>
-          <t>banner 744:464 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G55" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E56" s="10" t="inlineStr"/>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t>banner 745:477 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
-      <c r="J56" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3352,28 +3188,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>740:461</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="8" t="n">
+      <c r="A2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>742:459</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="8" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="G2" s="8" t="n">
-        <v>2</v>
+      <c r="F2" s="7" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
@@ -3381,28 +3217,28 @@
       <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>742:459</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7" t="n">
+      <c r="A3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>740:461</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F3" s="7" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>1</v>
+      <c r="F3" s="8" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
@@ -3410,28 +3246,28 @@
       <c r="K3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>740:463</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="8" t="n">
+      <c r="A4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>744:459</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="8" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>2</v>
+      <c r="F4" s="6" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
@@ -3439,28 +3275,28 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>744:459</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="6" t="n">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>740:463</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="6" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>0</v>
+      <c r="F5" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
@@ -3469,11 +3305,11 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>740:459</t>
+          <t>746:461</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
@@ -3486,7 +3322,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>17.3</v>
+        <v>12.7</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>1</v>
@@ -3515,7 +3351,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>13</v>
+        <v>14.2</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>1</v>
@@ -3527,11 +3363,11 @@
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>746:461</t>
+          <t>740:459</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
@@ -3544,7 +3380,7 @@
         <v>13</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>11.3</v>
+        <v>18.7</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>1</v>
@@ -3560,7 +3396,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>744:465</t>
+          <t>746:463</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
@@ -3573,7 +3409,7 @@
         <v>14</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>11.1</v>
+        <v>11.5</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>1</v>
@@ -3585,11 +3421,11 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>746:463</t>
+          <t>744:465</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -3602,7 +3438,7 @@
         <v>14</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>10.1</v>
+        <v>12.3</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>1</v>
@@ -3613,28 +3449,28 @@
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>740:465</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="8" t="n">
+      <c r="A11" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>746:459</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="8" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>2</v>
+      <c r="F11" s="6" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
@@ -3642,28 +3478,28 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>746:459</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6" t="n">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>740:465</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>0</v>
+      <c r="F12" s="8" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
@@ -3689,7 +3525,7 @@
         <v>16</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>1</v>
@@ -3700,28 +3536,28 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>738:461</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="8" t="n">
+      <c r="A14" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>742:457</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="8" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>2</v>
+      <c r="F14" s="7" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
@@ -3729,28 +3565,28 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>742:457</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="7" t="n">
+      <c r="A15" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>738:461</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>1</v>
+      <c r="F15" s="8" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -3758,28 +3594,28 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n">
-        <v>27</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>738:463</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="8" t="n">
+      <c r="A16" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>744:457</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F16" s="8" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>2</v>
+      <c r="F16" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -3787,28 +3623,28 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>744:457</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="6" t="n">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>738:463</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="F17" s="6" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>0</v>
+      <c r="F17" s="8" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -3817,11 +3653,11 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>738:459</t>
+          <t>740:457</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
@@ -3834,7 +3670,7 @@
         <v>17</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>19</v>
+        <v>19.9</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>1</v>
@@ -3846,11 +3682,11 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>740:457</t>
+          <t>738:459</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
@@ -3863,7 +3699,7 @@
         <v>17</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.5</v>
+        <v>20.4</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>1</v>
@@ -3874,28 +3710,28 @@
       <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n">
-        <v>37</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="A20" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>742:467</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="8" t="n">
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="8" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G20" s="8" t="n">
-        <v>2</v>
+      <c r="F20" s="7" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -3904,11 +3740,11 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>748:461</t>
+          <t>744:467</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
@@ -3921,7 +3757,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>9.9</v>
+        <v>11.8</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>1</v>
@@ -3933,7 +3769,7 @@
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
@@ -3950,7 +3786,7 @@
         <v>18</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>16.9</v>
+        <v>18.1</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>2</v>
@@ -3961,28 +3797,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
-        <v>43</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>744:467</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="F23" s="8" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>2</v>
+      <c r="A23" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>748:459</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -3991,11 +3827,11 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>748:463</t>
+          <t>746:467</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
@@ -4005,10 +3841,10 @@
         <v>2</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>8.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>1</v>
@@ -4019,28 +3855,28 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
-        <v>48</v>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>740:467</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="F25" s="8" t="n">
+      <c r="A25" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>748:457</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F25" s="6" t="n">
         <v>14.6</v>
       </c>
-      <c r="G25" s="8" t="n">
-        <v>2</v>
+      <c r="G25" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -4048,28 +3884,28 @@
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>748:459</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G26" s="6" t="n">
-        <v>0</v>
+      <c r="A26" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>748:467</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
@@ -4077,28 +3913,28 @@
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>746:467</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="8" t="n">
+      <c r="A27" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>742:455</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F27" s="8" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="G27" s="8" t="n">
-        <v>2</v>
+      <c r="F27" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -4106,28 +3942,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
-        <v>58</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>748:465</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="7" t="n">
+      <c r="A28" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>736:461</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="7" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <v>1</v>
+      <c r="F28" s="8" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -4135,28 +3971,28 @@
       <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n">
-        <v>68</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>738:467</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="G29" s="8" t="n">
-        <v>2</v>
+      <c r="A29" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>744:455</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
@@ -4164,28 +4000,28 @@
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>748:457</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>0</v>
+      <c r="A30" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>740:455</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
@@ -4194,24 +4030,24 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>748:467</t>
+          <t>736:459</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>6.7</v>
+        <v>22.1</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>1</v>
@@ -4222,28 +4058,28 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="n">
-        <v>52</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>736:461</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="8" t="n">
+      <c r="A32" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>746:455</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="G32" s="8" t="n">
-        <v>2</v>
+      <c r="E32" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -4251,28 +4087,28 @@
       <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n">
-        <v>54</v>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>742:455</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="7" t="n">
+      <c r="A33" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>736:465</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="7" t="n">
+      <c r="E33" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="F33" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F33" s="7" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>1</v>
+      <c r="G33" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -4280,28 +4116,28 @@
       <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>736:463</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="8" t="n">
+      <c r="A34" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>750:461</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E34" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F34" s="8" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G34" s="8" t="n">
-        <v>2</v>
+      <c r="E34" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
@@ -4309,28 +4145,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>744:455</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="6" t="n">
+      <c r="A35" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>742:469</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="G35" s="6" t="n">
-        <v>0</v>
+      <c r="E35" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -4338,28 +4174,28 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n">
-        <v>64</v>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>736:459</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="7" t="n">
+      <c r="A36" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>750:463</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="F36" s="7" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>1</v>
+      <c r="E36" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
@@ -4367,28 +4203,28 @@
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n">
-        <v>66</v>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>740:455</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="7" t="n">
+      <c r="A37" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>750:459</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="F37" s="7" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>1</v>
+      <c r="E37" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
@@ -4396,28 +4232,28 @@
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>746:455</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="6" t="n">
+      <c r="A38" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>738:455</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>0</v>
+      <c r="E38" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
@@ -4425,28 +4261,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
-        <v>75</v>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>750:461</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="6" t="n">
+      <c r="A39" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>736:457</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G39" s="6" t="n">
-        <v>0</v>
+      <c r="E39" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -4455,11 +4291,11 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>750:463</t>
+          <t>750:465</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
@@ -4469,7 +4305,7 @@
         <v>3</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>7.1</v>
@@ -4484,11 +4320,11 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>736:457</t>
+          <t>746:469</t>
         </is>
       </c>
       <c r="C41" s="7" t="n">
@@ -4498,10 +4334,10 @@
         <v>3</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>21.8</v>
+        <v>9.5</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>1</v>
@@ -4512,28 +4348,28 @@
       <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n">
-        <v>84</v>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>738:455</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="7" t="n">
+      <c r="A42" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>748:455</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E42" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="F42" s="7" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G42" s="7" t="n">
-        <v>1</v>
+      <c r="E42" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4" t="n"/>
@@ -4542,11 +4378,11 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>750:459</t>
+          <t>750:457</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
@@ -4556,10 +4392,10 @@
         <v>3</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>10.5</v>
+        <v>13.7</v>
       </c>
       <c r="G43" s="6" t="n">
         <v>0</v>
@@ -4570,28 +4406,28 @@
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="n">
-        <v>89</v>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>746:469</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="8" t="n">
+      <c r="A44" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>736:455</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="F44" s="8" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G44" s="8" t="n">
-        <v>2</v>
+      <c r="E44" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
@@ -4599,28 +4435,28 @@
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
-        <v>91</v>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>750:465</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="6" t="n">
+      <c r="A45" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>748:469</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="F45" s="6" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="G45" s="6" t="n">
-        <v>0</v>
+      <c r="E45" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F45" s="7" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
@@ -4629,24 +4465,24 @@
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>736:467</t>
+          <t>734:461</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E46" s="8" t="n">
         <v>25</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>18.6</v>
+        <v>23.1</v>
       </c>
       <c r="G46" s="8" t="n">
         <v>2</v>
@@ -4658,24 +4494,24 @@
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>748:455</t>
+          <t>744:453</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>15</v>
+        <v>20.1</v>
       </c>
       <c r="G47" s="6" t="n">
         <v>0</v>
@@ -4686,28 +4522,28 @@
       <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
-        <v>96</v>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>750:457</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E48" s="6" t="n">
+      <c r="A48" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>734:463</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="F48" s="6" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>0</v>
+      <c r="F48" s="8" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G48" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
@@ -4715,28 +4551,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
-        <v>98</v>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>736:455</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="7" t="n">
+      <c r="A49" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>746:453</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="F49" s="7" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="G49" s="7" t="n">
-        <v>1</v>
+      <c r="F49" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -4744,28 +4580,28 @@
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>750:467</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E50" s="6" t="n">
+      <c r="A50" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>734:465</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="F50" s="6" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>0</v>
+      <c r="F50" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
@@ -4773,28 +4609,28 @@
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>740:477</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="9" t="n">
+      <c r="A51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>742:475</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F51" s="9" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <v>3</v>
+      <c r="F51" s="6" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
@@ -4803,11 +4639,11 @@
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>742:475</t>
+          <t>740:477</t>
         </is>
       </c>
       <c r="C52" s="7" t="n">
@@ -4820,7 +4656,7 @@
         <v>10</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>14.1</v>
+        <v>17.2</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>1</v>
@@ -4831,28 +4667,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>740:479</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="9" t="n">
+      <c r="A53" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>744:475</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F53" s="9" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <v>3</v>
+      <c r="F53" s="6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G53" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4865,7 +4701,7 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>744:475</t>
+          <t>740:479</t>
         </is>
       </c>
       <c r="C54" s="7" t="n">
@@ -4878,7 +4714,7 @@
         <v>11</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>12.3</v>
+        <v>18.2</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>1</v>
@@ -4889,28 +4725,28 @@
       <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>740:475</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="8" t="n">
+      <c r="A55" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>746:477</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F55" s="8" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="G55" s="8" t="n">
-        <v>2</v>
+      <c r="F55" s="6" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -4918,28 +4754,28 @@
       <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n">
+      <c r="A56" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>742:481</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="8" t="n">
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>740:475</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F56" s="8" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G56" s="8" t="n">
-        <v>2</v>
+      <c r="F56" s="7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G56" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
@@ -4947,28 +4783,28 @@
       <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>746:477</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="7" t="n">
+      <c r="A57" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F57" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="G57" s="7" t="n">
-        <v>1</v>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>742:481</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -4976,28 +4812,28 @@
       <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>744:481</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="8" t="n">
+      <c r="A58" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>746:479</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F58" s="8" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="G58" s="8" t="n">
-        <v>2</v>
+      <c r="F58" s="6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
@@ -5005,28 +4841,28 @@
       <c r="K58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="n">
+      <c r="A59" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>746:479</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="7" t="n">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>744:481</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F59" s="7" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="G59" s="7" t="n">
-        <v>1</v>
+      <c r="F59" s="6" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H59" s="4" t="n"/>
       <c r="I59" s="4" t="n"/>
@@ -5034,28 +4870,28 @@
       <c r="K59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>740:481</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="9" t="n">
+      <c r="A60" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>746:475</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F60" s="9" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>3</v>
+      <c r="F60" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
@@ -5068,7 +4904,7 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>746:475</t>
+          <t>740:481</t>
         </is>
       </c>
       <c r="C61" s="7" t="n">
@@ -5081,7 +4917,7 @@
         <v>15</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>10.7</v>
+        <v>19.3</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>1</v>
@@ -5092,28 +4928,28 @@
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="n">
+      <c r="A62" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>746:481</t>
         </is>
       </c>
-      <c r="C62" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="8" t="n">
+      <c r="C62" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F62" s="8" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="G62" s="8" t="n">
-        <v>2</v>
+      <c r="F62" s="6" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G62" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
@@ -5121,28 +4957,28 @@
       <c r="K62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>738:477</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="9" t="n">
+      <c r="A63" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>742:473</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F63" s="9" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G63" s="9" t="n">
-        <v>3</v>
+      <c r="F63" s="7" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
@@ -5150,28 +4986,28 @@
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>742:473</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E64" s="8" t="n">
+      <c r="A64" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>738:477</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F64" s="8" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="G64" s="8" t="n">
-        <v>2</v>
+      <c r="F64" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
@@ -5179,28 +5015,28 @@
       <c r="K64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>738:479</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="9" t="n">
+      <c r="A65" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>744:473</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="F65" s="9" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G65" s="9" t="n">
-        <v>3</v>
+      <c r="F65" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G65" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
@@ -5208,28 +5044,28 @@
       <c r="K65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="n">
+      <c r="A66" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>744:473</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" s="8" t="n">
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>738:479</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="F66" s="8" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="G66" s="8" t="n">
-        <v>2</v>
+      <c r="F66" s="7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
@@ -5237,28 +5073,28 @@
       <c r="K66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="n">
-        <v>34</v>
-      </c>
-      <c r="B67" s="8" t="inlineStr">
-        <is>
-          <t>738:475</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" s="8" t="n">
+      <c r="A67" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>740:473</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="F67" s="8" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G67" s="8" t="n">
-        <v>2</v>
+      <c r="F67" s="7" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
@@ -5266,28 +5102,28 @@
       <c r="K67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>740:473</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E68" s="8" t="n">
+      <c r="A68" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>738:475</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="F68" s="8" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="G68" s="8" t="n">
-        <v>2</v>
+      <c r="F68" s="7" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
@@ -5295,28 +5131,28 @@
       <c r="K68" s="4" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>742:483</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D69" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E69" s="8" t="n">
+      <c r="A69" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>748:477</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F69" s="8" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="G69" s="8" t="n">
-        <v>2</v>
+      <c r="F69" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G69" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
@@ -5324,28 +5160,28 @@
       <c r="K69" s="4" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="B70" s="7" t="inlineStr">
-        <is>
-          <t>748:477</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D70" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E70" s="7" t="n">
+      <c r="A70" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>742:483</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E70" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F70" s="7" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="G70" s="7" t="n">
-        <v>1</v>
+      <c r="F70" s="6" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G70" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
@@ -5353,28 +5189,28 @@
       <c r="K70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="B71" s="9" t="inlineStr">
-        <is>
-          <t>738:481</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" s="9" t="n">
+      <c r="A71" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>746:473</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F71" s="9" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="G71" s="9" t="n">
-        <v>3</v>
+      <c r="F71" s="7" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G71" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
@@ -5382,28 +5218,28 @@
       <c r="K71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>744:483</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" s="8" t="n">
+      <c r="A72" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>748:479</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F72" s="8" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G72" s="8" t="n">
-        <v>2</v>
+      <c r="F72" s="7" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
@@ -5411,28 +5247,28 @@
       <c r="K72" s="4" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>746:473</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="8" t="n">
+      <c r="A73" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>744:483</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F73" s="8" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G73" s="8" t="n">
-        <v>2</v>
+      <c r="F73" s="6" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G73" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="n"/>
@@ -5441,11 +5277,11 @@
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>748:479</t>
+          <t>738:481</t>
         </is>
       </c>
       <c r="C74" s="7" t="n">
@@ -5458,7 +5294,7 @@
         <v>18</v>
       </c>
       <c r="F74" s="7" t="n">
-        <v>12.3</v>
+        <v>20.9</v>
       </c>
       <c r="G74" s="7" t="n">
         <v>1</v>
@@ -5469,28 +5305,28 @@
       <c r="K74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>49</v>
-      </c>
-      <c r="B75" s="9" t="inlineStr">
-        <is>
-          <t>740:483</t>
-        </is>
-      </c>
-      <c r="C75" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D75" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" s="9" t="n">
+      <c r="A75" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>748:475</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="F75" s="9" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="G75" s="9" t="n">
-        <v>3</v>
+      <c r="F75" s="6" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="G75" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
@@ -5499,11 +5335,11 @@
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>748:475</t>
+          <t>740:483</t>
         </is>
       </c>
       <c r="C76" s="7" t="n">
@@ -5516,7 +5352,7 @@
         <v>19</v>
       </c>
       <c r="F76" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>20.6</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>1</v>
@@ -5528,11 +5364,11 @@
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>746:483</t>
+          <t>748:481</t>
         </is>
       </c>
       <c r="C77" s="7" t="n">
@@ -5545,7 +5381,7 @@
         <v>20</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>16.8</v>
+        <v>13.7</v>
       </c>
       <c r="G77" s="7" t="n">
         <v>1</v>
@@ -5557,11 +5393,11 @@
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>748:481</t>
+          <t>746:483</t>
         </is>
       </c>
       <c r="C78" s="7" t="n">
@@ -5574,7 +5410,7 @@
         <v>20</v>
       </c>
       <c r="F78" s="7" t="n">
-        <v>14.1</v>
+        <v>16.5</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>1</v>
@@ -5585,28 +5421,28 @@
       <c r="K78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="9" t="n">
-        <v>69</v>
-      </c>
-      <c r="B79" s="9" t="inlineStr">
-        <is>
-          <t>738:483</t>
-        </is>
-      </c>
-      <c r="C79" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D79" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" s="9" t="n">
+      <c r="A79" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>748:473</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F79" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="G79" s="9" t="n">
-        <v>3</v>
+      <c r="F79" s="7" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
@@ -5615,11 +5451,11 @@
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>748:473</t>
+          <t>748:483</t>
         </is>
       </c>
       <c r="C80" s="7" t="n">
@@ -5629,10 +5465,10 @@
         <v>2</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F80" s="7" t="n">
-        <v>7.9</v>
+        <v>15.4</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>1</v>
@@ -5644,24 +5480,24 @@
     </row>
     <row r="81">
       <c r="A81" s="7" t="n">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>748:483</t>
+          <t>742:471</t>
         </is>
       </c>
       <c r="C81" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>15.9</v>
+        <v>13.6</v>
       </c>
       <c r="G81" s="7" t="n">
         <v>1</v>
@@ -5672,28 +5508,28 @@
       <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="n">
-        <v>53</v>
-      </c>
-      <c r="B82" s="9" t="inlineStr">
+      <c r="A82" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>736:477</t>
         </is>
       </c>
-      <c r="C82" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="9" t="n">
+      <c r="C82" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E82" s="9" t="n">
+      <c r="E82" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F82" s="9" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G82" s="9" t="n">
-        <v>3</v>
+      <c r="F82" s="7" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
@@ -5701,28 +5537,28 @@
       <c r="K82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>742:471</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D83" s="8" t="n">
+      <c r="A83" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>744:471</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E83" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F83" s="8" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G83" s="8" t="n">
-        <v>2</v>
+      <c r="E83" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="F83" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G83" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H83" s="4" t="n"/>
       <c r="I83" s="4" t="n"/>
@@ -5730,28 +5566,28 @@
       <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="B84" s="9" t="inlineStr">
-        <is>
-          <t>736:479</t>
-        </is>
-      </c>
-      <c r="C84" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="9" t="n">
+      <c r="A84" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>740:471</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="9" t="n">
+      <c r="E84" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F84" s="9" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G84" s="9" t="n">
-        <v>3</v>
+      <c r="F84" s="7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
@@ -5759,28 +5595,28 @@
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="n">
-        <v>63</v>
-      </c>
-      <c r="B85" s="8" t="inlineStr">
-        <is>
-          <t>744:471</t>
-        </is>
-      </c>
-      <c r="C85" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="8" t="n">
+      <c r="A85" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>736:475</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E85" s="8" t="n">
+      <c r="E85" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F85" s="8" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="G85" s="8" t="n">
-        <v>2</v>
+      <c r="F85" s="7" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="G85" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
@@ -5788,28 +5624,28 @@
       <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
-        <is>
-          <t>736:475</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="8" t="n">
+      <c r="A86" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>746:471</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E86" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F86" s="8" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G86" s="8" t="n">
-        <v>2</v>
+      <c r="E86" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F86" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G86" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -5817,28 +5653,28 @@
       <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="n">
+      <c r="A87" s="7" t="n">
         <v>67</v>
       </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>740:471</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="8" t="n">
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>736:481</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E87" s="8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F87" s="8" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="G87" s="8" t="n">
-        <v>2</v>
+      <c r="E87" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F87" s="7" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G87" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H87" s="4" t="n"/>
       <c r="I87" s="4" t="n"/>
@@ -5846,28 +5682,28 @@
       <c r="K87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="n">
-        <v>73</v>
-      </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t>746:471</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="8" t="n">
+      <c r="A88" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>750:477</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E88" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="F88" s="8" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G88" s="8" t="n">
-        <v>2</v>
+      <c r="E88" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F88" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="G88" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H88" s="4" t="n"/>
       <c r="I88" s="4" t="n"/>
@@ -5875,28 +5711,28 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="A89" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>742:485</t>
         </is>
       </c>
-      <c r="C89" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D89" s="8" t="n">
+      <c r="C89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E89" s="8" t="n">
+      <c r="E89" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F89" s="8" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="G89" s="8" t="n">
-        <v>2</v>
+      <c r="F89" s="6" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G89" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
@@ -5905,11 +5741,11 @@
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>750:477</t>
+          <t>750:479</t>
         </is>
       </c>
       <c r="C90" s="7" t="n">
@@ -5922,7 +5758,7 @@
         <v>23</v>
       </c>
       <c r="F90" s="7" t="n">
-        <v>9.6</v>
+        <v>11</v>
       </c>
       <c r="G90" s="7" t="n">
         <v>1</v>
@@ -5933,28 +5769,28 @@
       <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="n">
-        <v>77</v>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="A91" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>744:485</t>
         </is>
       </c>
-      <c r="C91" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D91" s="8" t="n">
+      <c r="C91" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E91" s="8" t="n">
+      <c r="E91" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F91" s="8" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G91" s="8" t="n">
-        <v>2</v>
+      <c r="F91" s="6" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G91" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H91" s="4" t="n"/>
       <c r="I91" s="4" t="n"/>
@@ -5962,28 +5798,28 @@
       <c r="K91" s="4" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
-        <is>
-          <t>750:479</t>
-        </is>
-      </c>
-      <c r="C92" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D92" s="7" t="n">
+      <c r="A92" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>750:475</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E92" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="F92" s="7" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="G92" s="7" t="n">
-        <v>1</v>
+      <c r="E92" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G92" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H92" s="4" t="n"/>
       <c r="I92" s="4" t="n"/>
@@ -5991,28 +5827,28 @@
       <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="n">
-        <v>83</v>
-      </c>
-      <c r="B93" s="8" t="inlineStr">
-        <is>
-          <t>736:473</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="8" t="n">
+      <c r="A93" s="7" t="n">
+        <v>79</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>738:471</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E93" s="8" t="n">
+      <c r="E93" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="F93" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="G93" s="8" t="n">
-        <v>2</v>
+      <c r="F93" s="7" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G93" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H93" s="4" t="n"/>
       <c r="I93" s="4" t="n"/>
@@ -6020,28 +5856,28 @@
       <c r="K93" s="4" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="B94" s="8" t="inlineStr">
-        <is>
-          <t>738:471</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D94" s="8" t="n">
+      <c r="A94" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>736:473</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E94" s="8" t="n">
+      <c r="E94" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="F94" s="8" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="G94" s="8" t="n">
-        <v>2</v>
+      <c r="F94" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G94" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H94" s="4" t="n"/>
       <c r="I94" s="4" t="n"/>
@@ -6049,28 +5885,28 @@
       <c r="K94" s="4" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="n">
-        <v>86</v>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="A95" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
         <is>
           <t>740:485</t>
         </is>
       </c>
-      <c r="C95" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D95" s="8" t="n">
+      <c r="C95" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E95" s="8" t="n">
+      <c r="E95" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="F95" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="G95" s="8" t="n">
-        <v>2</v>
+      <c r="F95" s="6" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="G95" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H95" s="4" t="n"/>
       <c r="I95" s="4" t="n"/>
@@ -6078,28 +5914,28 @@
       <c r="K95" s="4" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="6" t="n">
-        <v>88</v>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>750:475</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="6" t="n">
+      <c r="A96" s="7" t="n">
+        <v>86</v>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>748:471</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="F96" s="6" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="G96" s="6" t="n">
-        <v>0</v>
+      <c r="E96" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F96" s="7" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G96" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H96" s="4" t="n"/>
       <c r="I96" s="4" t="n"/>
@@ -6107,28 +5943,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>746:485</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="7" t="n">
+      <c r="A97" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>750:473</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="F97" s="7" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G97" s="7" t="n">
-        <v>1</v>
+      <c r="E97" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G97" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
@@ -6137,11 +5973,11 @@
     </row>
     <row r="98">
       <c r="A98" s="7" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>750:481</t>
+          <t>736:471</t>
         </is>
       </c>
       <c r="C98" s="7" t="n">
@@ -6151,10 +5987,10 @@
         <v>3</v>
       </c>
       <c r="E98" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F98" s="7" t="n">
-        <v>13.3</v>
+        <v>19.6</v>
       </c>
       <c r="G98" s="7" t="n">
         <v>1</v>
@@ -6166,24 +6002,24 @@
     </row>
     <row r="99">
       <c r="A99" s="7" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>748:471</t>
+          <t>734:477</t>
         </is>
       </c>
       <c r="C99" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E99" s="7" t="n">
         <v>25</v>
       </c>
       <c r="F99" s="7" t="n">
-        <v>7</v>
+        <v>22.8</v>
       </c>
       <c r="G99" s="7" t="n">
         <v>1</v>
@@ -6194,28 +6030,28 @@
       <c r="K99" s="4" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="n">
-        <v>97</v>
-      </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>750:473</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E100" s="6" t="n">
+      <c r="A100" s="7" t="n">
+        <v>92</v>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>734:479</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E100" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="F100" s="6" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="G100" s="6" t="n">
-        <v>0</v>
+      <c r="F100" s="7" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="G100" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H100" s="4" t="n"/>
       <c r="I100" s="4" t="n"/>
@@ -6223,28 +6059,28 @@
       <c r="K100" s="4" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="n">
+      <c r="A101" s="7" t="n">
         <v>99</v>
       </c>
-      <c r="B101" s="8" t="inlineStr">
-        <is>
-          <t>736:471</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D101" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E101" s="8" t="n">
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>734:481</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E101" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="F101" s="8" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G101" s="8" t="n">
-        <v>2</v>
+      <c r="F101" s="7" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="G101" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H101" s="4" t="n"/>
       <c r="I101" s="4" t="n"/>

</xml_diff>

<commit_message>
Design of 19 Sep night: rings 1-3 only, no holes, 9 new banners (3 built stay); HQ territory at x 749-763, y 463-477
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -1422,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>739:457</t>
+          <t>737:483</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>11 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H44" s="4" t="n"/>
@@ -2830,7 +2830,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>744:464</t>
+          <t>738:476</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Trap 1 site 743:462; 5 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H45" s="4" t="n"/>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>745:470</t>
+          <t>739:456</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>15 slots (file order)</t>
+          <t>6 slots (file order)</t>
         </is>
       </c>
       <c r="H46" s="4" t="n"/>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>738:473</t>
+          <t>741:470</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>8 slots (file order)</t>
+          <t>9 slots (file order)</t>
         </is>
       </c>
       <c r="H47" s="4" t="n"/>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>737:480</t>
+          <t>745:463</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>12 slots (file order)</t>
+          <t>Trap 1 site 743:462; 8 slots (file order)</t>
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>750:481</t>
+          <t>748:470</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H49" s="4" t="n"/>
@@ -3000,35 +3000,35 @@
       <c r="J49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="7" t="n">
         <v>48</v>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>737:463</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="n">
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>750:481</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G50" s="8" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>7 slots (file order)</t>
         </is>
       </c>
       <c r="H50" s="4" t="n"/>
@@ -3036,33 +3036,35 @@
       <c r="J50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="n">
+      <c r="A51" s="7" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr"/>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>banner 744:464 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>752:459</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
@@ -3070,38 +3072,108 @@
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n">
+      <c r="A52" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr"/>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>banner 745:477 (built); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>738:463</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>wave 2</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>wave 1 complete</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
       <c r="J52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr"/>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>banner 745:463 (wave 1); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr"/>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>banner 745:477 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
+      <c r="J54" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3362,28 +3434,28 @@
       <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>740:459</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="n">
+      <c r="C8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>18.7</v>
       </c>
-      <c r="G8" s="7" t="n">
-        <v>1</v>
+      <c r="G8" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
@@ -3508,7 +3580,7 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
@@ -3623,28 +3695,28 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n">
-        <v>29</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>738:463</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>2</v>
+      <c r="A17" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>740:457</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -3652,28 +3724,28 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>740:457</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="7" t="n">
+      <c r="A18" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>738:459</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="F18" s="7" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>1</v>
+      <c r="F18" s="8" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
@@ -3686,7 +3758,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>738:459</t>
+          <t>748:461</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
@@ -3696,10 +3768,10 @@
         <v>2</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>20.4</v>
+        <v>11.3</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>1</v>
@@ -3711,7 +3783,7 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
@@ -3740,11 +3812,11 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>744:467</t>
+          <t>748:463</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
@@ -3757,7 +3829,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>11.8</v>
+        <v>9.9</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>1</v>
@@ -3768,28 +3840,28 @@
       <c r="K21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>738:465</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="8" t="n">
+      <c r="A22" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>744:467</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="8" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>2</v>
+      <c r="F22" s="7" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
@@ -3797,28 +3869,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>748:459</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>0</v>
+      <c r="A23" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>738:465</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -3826,28 +3898,28 @@
       <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n">
-        <v>49</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>746:467</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F24" s="7" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
+      <c r="A24" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>748:459</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -3855,28 +3927,28 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>63</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>748:457</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>0</v>
+      <c r="A25" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>740:467</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -3885,11 +3957,11 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>748:467</t>
+          <t>738:457</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
@@ -3899,10 +3971,10 @@
         <v>2</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>7.9</v>
+        <v>21.5</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>1</v>
@@ -3914,24 +3986,24 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>742:455</t>
+          <t>748:465</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>20</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>19.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>1</v>
@@ -3942,28 +4014,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>736:461</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E28" s="8" t="n">
+      <c r="A28" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>746:467</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="8" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G28" s="8" t="n">
-        <v>2</v>
+      <c r="F28" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -3972,24 +4044,24 @@
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>744:455</t>
+          <t>748:457</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>18.5</v>
+        <v>14.6</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>0</v>
@@ -4001,24 +4073,24 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>740:455</t>
+          <t>738:467</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>21.2</v>
+        <v>17.7</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>1</v>
@@ -4030,24 +4102,24 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>736:459</t>
+          <t>748:467</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>22.1</v>
+        <v>7.9</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>1</v>
@@ -4058,28 +4130,28 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>65</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>746:455</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="6" t="n">
+      <c r="A32" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>742:455</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>0</v>
+      <c r="E32" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -4088,11 +4160,11 @@
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>736:465</t>
+          <t>736:461</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
@@ -4102,10 +4174,10 @@
         <v>3</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>20</v>
+        <v>21.3</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>2</v>
@@ -4117,11 +4189,11 @@
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>750:461</t>
+          <t>744:455</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
@@ -4131,10 +4203,10 @@
         <v>3</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>10.1</v>
+        <v>18.5</v>
       </c>
       <c r="G34" s="6" t="n">
         <v>0</v>
@@ -4145,28 +4217,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>742:469</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="7" t="n">
+      <c r="A35" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>736:463</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>1</v>
+      <c r="E35" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -4174,28 +4246,28 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n">
-        <v>72</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>750:463</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="6" t="n">
+      <c r="A36" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>740:455</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G36" s="6" t="n">
-        <v>0</v>
+      <c r="E36" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
@@ -4203,28 +4275,28 @@
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n">
-        <v>78</v>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>750:459</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="6" t="n">
+      <c r="A37" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>736:459</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>0</v>
+      <c r="E37" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
@@ -4232,28 +4304,28 @@
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n">
-        <v>82</v>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>738:455</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="7" t="n">
+      <c r="A38" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>746:455</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="F38" s="7" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="G38" s="7" t="n">
-        <v>1</v>
+      <c r="E38" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n"/>
@@ -4261,28 +4333,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n">
-        <v>83</v>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>736:457</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="7" t="n">
+      <c r="A39" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>736:465</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="F39" s="7" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>1</v>
+      <c r="E39" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -4291,11 +4363,11 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>750:465</t>
+          <t>750:461</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
@@ -4305,10 +4377,10 @@
         <v>3</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>7.1</v>
+        <v>10.1</v>
       </c>
       <c r="G40" s="6" t="n">
         <v>0</v>
@@ -4320,11 +4392,11 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>746:469</t>
+          <t>742:469</t>
         </is>
       </c>
       <c r="C41" s="7" t="n">
@@ -4334,10 +4406,10 @@
         <v>3</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>9.5</v>
+        <v>13.5</v>
       </c>
       <c r="G41" s="7" t="n">
         <v>1</v>
@@ -4349,11 +4421,11 @@
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>748:455</t>
+          <t>750:463</t>
         </is>
       </c>
       <c r="C42" s="6" t="n">
@@ -4363,10 +4435,10 @@
         <v>3</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>16.3</v>
+        <v>8.5</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>0</v>
@@ -4377,28 +4449,28 @@
       <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n">
-        <v>94</v>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>750:457</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="6" t="n">
+      <c r="A43" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>744:469</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F43" s="6" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G43" s="6" t="n">
-        <v>0</v>
+      <c r="E43" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
@@ -4406,28 +4478,28 @@
       <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
-        <v>98</v>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>736:455</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="7" t="n">
+      <c r="A44" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>750:459</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="F44" s="7" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="G44" s="7" t="n">
-        <v>1</v>
+      <c r="E44" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4" t="n"/>
@@ -4436,11 +4508,11 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>748:469</t>
+          <t>736:457</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
@@ -4450,10 +4522,10 @@
         <v>3</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>7.5</v>
+        <v>23.2</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>1</v>
@@ -4464,28 +4536,28 @@
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="n">
-        <v>89</v>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>734:461</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E46" s="8" t="n">
+      <c r="A46" s="6" t="n">
+        <v>92</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>750:465</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F46" s="8" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="G46" s="8" t="n">
-        <v>2</v>
+      <c r="F46" s="6" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4" t="n"/>
@@ -4493,28 +4565,28 @@
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>744:453</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E47" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="G47" s="6" t="n">
-        <v>0</v>
+      <c r="A47" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>746:469</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F47" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
@@ -4522,28 +4594,28 @@
       <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>734:463</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E48" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="F48" s="8" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="G48" s="8" t="n">
-        <v>2</v>
+      <c r="A48" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>748:455</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
@@ -4551,28 +4623,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>746:453</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="G49" s="6" t="n">
-        <v>0</v>
+      <c r="A49" s="7" t="n">
+        <v>97</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>738:469</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F49" s="7" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -4580,28 +4652,28 @@
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>734:465</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="8" t="n">
+      <c r="A50" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>750:467</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="F50" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="G50" s="8" t="n">
-        <v>2</v>
+      <c r="F50" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
@@ -4610,24 +4682,24 @@
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>742:475</t>
+          <t>750:469</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>14.6</v>
+        <v>5.5</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
@@ -4638,28 +4710,28 @@
       <c r="K51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>740:477</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="7" t="n">
+      <c r="A52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>742:475</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F52" s="7" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>1</v>
+      <c r="F52" s="6" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
@@ -4667,28 +4739,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>744:475</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>0</v>
+      <c r="A53" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>740:477</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F53" s="7" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G53" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4696,28 +4768,28 @@
       <c r="K53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>740:479</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="7" t="n">
+      <c r="A54" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>744:475</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F54" s="7" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="G54" s="7" t="n">
-        <v>1</v>
+      <c r="F54" s="6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
@@ -4725,28 +4797,28 @@
       <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>746:477</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>0</v>
+      <c r="A55" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>740:479</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -4754,28 +4826,28 @@
       <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>740:475</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="7" t="n">
+      <c r="A56" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>746:477</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F56" s="7" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="G56" s="7" t="n">
-        <v>1</v>
+      <c r="F56" s="6" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
@@ -4783,28 +4855,28 @@
       <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n">
+      <c r="A57" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>740:475</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>742:481</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>0</v>
+      <c r="F57" s="7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -4813,11 +4885,11 @@
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>746:479</t>
+          <t>742:481</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
@@ -4827,10 +4899,10 @@
         <v>1</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>13.4</v>
+        <v>17.7</v>
       </c>
       <c r="G58" s="6" t="n">
         <v>0</v>
@@ -4842,11 +4914,11 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>744:481</t>
+          <t>746:479</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
@@ -4859,7 +4931,7 @@
         <v>14</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>16.3</v>
+        <v>13.4</v>
       </c>
       <c r="G59" s="6" t="n">
         <v>0</v>
@@ -4871,11 +4943,11 @@
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>746:475</t>
+          <t>744:481</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
@@ -4885,10 +4957,10 @@
         <v>1</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>11</v>
+        <v>16.3</v>
       </c>
       <c r="G60" s="6" t="n">
         <v>0</v>
@@ -4899,28 +4971,28 @@
       <c r="K60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>740:481</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D61" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="7" t="n">
+      <c r="A61" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>746:475</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F61" s="7" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G61" s="7" t="n">
-        <v>1</v>
+      <c r="F61" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
@@ -4928,28 +5000,28 @@
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>746:481</t>
-        </is>
-      </c>
-      <c r="C62" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="F62" s="6" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="G62" s="6" t="n">
-        <v>0</v>
+      <c r="A62" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>740:481</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F62" s="7" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G62" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
@@ -4957,28 +5029,28 @@
       <c r="K62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B63" s="7" t="inlineStr">
-        <is>
-          <t>742:473</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="F63" s="7" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="G63" s="7" t="n">
-        <v>1</v>
+      <c r="A63" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>746:481</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
@@ -4987,11 +5059,11 @@
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>738:477</t>
+          <t>742:473</t>
         </is>
       </c>
       <c r="C64" s="7" t="n">
@@ -5004,7 +5076,7 @@
         <v>15</v>
       </c>
       <c r="F64" s="7" t="n">
-        <v>19</v>
+        <v>13.9</v>
       </c>
       <c r="G64" s="7" t="n">
         <v>1</v>
@@ -5016,11 +5088,11 @@
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>744:473</t>
+          <t>738:477</t>
         </is>
       </c>
       <c r="C65" s="7" t="n">
@@ -5030,10 +5102,10 @@
         <v>2</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G65" s="7" t="n">
         <v>1</v>
@@ -5045,11 +5117,11 @@
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>738:479</t>
+          <t>744:473</t>
         </is>
       </c>
       <c r="C66" s="7" t="n">
@@ -5062,7 +5134,7 @@
         <v>16</v>
       </c>
       <c r="F66" s="7" t="n">
-        <v>19.9</v>
+        <v>12</v>
       </c>
       <c r="G66" s="7" t="n">
         <v>1</v>
@@ -5074,11 +5146,11 @@
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>740:473</t>
+          <t>738:479</t>
         </is>
       </c>
       <c r="C67" s="7" t="n">
@@ -5088,10 +5160,10 @@
         <v>2</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>15.9</v>
+        <v>19.9</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>1</v>
@@ -5103,11 +5175,11 @@
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>738:475</t>
+          <t>740:473</t>
         </is>
       </c>
       <c r="C68" s="7" t="n">
@@ -5120,7 +5192,7 @@
         <v>17</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>18.3</v>
+        <v>15.9</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>1</v>
@@ -5132,7 +5204,7 @@
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
@@ -5161,7 +5233,7 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
@@ -5335,7 +5407,7 @@
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
@@ -5364,11 +5436,11 @@
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>748:481</t>
+          <t>738:473</t>
         </is>
       </c>
       <c r="C77" s="7" t="n">
@@ -5381,7 +5453,7 @@
         <v>20</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>13.7</v>
+        <v>17.8</v>
       </c>
       <c r="G77" s="7" t="n">
         <v>1</v>
@@ -5393,11 +5465,11 @@
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>746:483</t>
+          <t>748:481</t>
         </is>
       </c>
       <c r="C78" s="7" t="n">
@@ -5410,7 +5482,7 @@
         <v>20</v>
       </c>
       <c r="F78" s="7" t="n">
-        <v>16.5</v>
+        <v>13.7</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>1</v>
@@ -5422,11 +5494,11 @@
     </row>
     <row r="79">
       <c r="A79" s="7" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>748:473</t>
+          <t>746:483</t>
         </is>
       </c>
       <c r="C79" s="7" t="n">
@@ -5436,10 +5508,10 @@
         <v>2</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>8.300000000000001</v>
+        <v>16.5</v>
       </c>
       <c r="G79" s="7" t="n">
         <v>1</v>
@@ -5451,11 +5523,11 @@
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>748:483</t>
+          <t>748:473</t>
         </is>
       </c>
       <c r="C80" s="7" t="n">
@@ -5465,10 +5537,10 @@
         <v>2</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F80" s="7" t="n">
-        <v>15.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>1</v>
@@ -5480,24 +5552,24 @@
     </row>
     <row r="81">
       <c r="A81" s="7" t="n">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>742:471</t>
+          <t>738:483</t>
         </is>
       </c>
       <c r="C81" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>13.6</v>
+        <v>22.1</v>
       </c>
       <c r="G81" s="7" t="n">
         <v>1</v>
@@ -5509,24 +5581,24 @@
     </row>
     <row r="82">
       <c r="A82" s="7" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>736:477</t>
+          <t>748:483</t>
         </is>
       </c>
       <c r="C82" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>20.9</v>
+        <v>15.4</v>
       </c>
       <c r="G82" s="7" t="n">
         <v>1</v>
@@ -5538,11 +5610,11 @@
     </row>
     <row r="83">
       <c r="A83" s="7" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>744:471</t>
+          <t>742:471</t>
         </is>
       </c>
       <c r="C83" s="7" t="n">
@@ -5552,10 +5624,10 @@
         <v>3</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F83" s="7" t="n">
-        <v>11.6</v>
+        <v>13.6</v>
       </c>
       <c r="G83" s="7" t="n">
         <v>1</v>
@@ -5571,7 +5643,7 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>740:471</t>
+          <t>736:477</t>
         </is>
       </c>
       <c r="C84" s="7" t="n">
@@ -5581,10 +5653,10 @@
         <v>3</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F84" s="7" t="n">
-        <v>15.6</v>
+        <v>20.9</v>
       </c>
       <c r="G84" s="7" t="n">
         <v>1</v>
@@ -5596,11 +5668,11 @@
     </row>
     <row r="85">
       <c r="A85" s="7" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>736:475</t>
+          <t>744:471</t>
         </is>
       </c>
       <c r="C85" s="7" t="n">
@@ -5613,7 +5685,7 @@
         <v>21</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>20.3</v>
+        <v>11.6</v>
       </c>
       <c r="G85" s="7" t="n">
         <v>1</v>
@@ -5625,11 +5697,11 @@
     </row>
     <row r="86">
       <c r="A86" s="7" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>746:471</t>
+          <t>736:479</t>
         </is>
       </c>
       <c r="C86" s="7" t="n">
@@ -5639,10 +5711,10 @@
         <v>3</v>
       </c>
       <c r="E86" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F86" s="7" t="n">
-        <v>9.6</v>
+        <v>21.7</v>
       </c>
       <c r="G86" s="7" t="n">
         <v>1</v>
@@ -5654,11 +5726,11 @@
     </row>
     <row r="87">
       <c r="A87" s="7" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>736:481</t>
+          <t>740:471</t>
         </is>
       </c>
       <c r="C87" s="7" t="n">
@@ -5668,10 +5740,10 @@
         <v>3</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F87" s="7" t="n">
-        <v>22.6</v>
+        <v>15.6</v>
       </c>
       <c r="G87" s="7" t="n">
         <v>1</v>
@@ -5683,11 +5755,11 @@
     </row>
     <row r="88">
       <c r="A88" s="7" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>750:477</t>
+          <t>736:475</t>
         </is>
       </c>
       <c r="C88" s="7" t="n">
@@ -5697,10 +5769,10 @@
         <v>3</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F88" s="7" t="n">
-        <v>9.300000000000001</v>
+        <v>20.3</v>
       </c>
       <c r="G88" s="7" t="n">
         <v>1</v>
@@ -5711,28 +5783,28 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="6" t="n">
-        <v>71</v>
-      </c>
-      <c r="B89" s="6" t="inlineStr">
-        <is>
-          <t>742:485</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D89" s="6" t="n">
+      <c r="A89" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>746:471</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E89" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F89" s="6" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="G89" s="6" t="n">
-        <v>0</v>
+      <c r="E89" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F89" s="7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G89" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
@@ -5741,11 +5813,11 @@
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>750:479</t>
+          <t>736:481</t>
         </is>
       </c>
       <c r="C90" s="7" t="n">
@@ -5755,10 +5827,10 @@
         <v>3</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F90" s="7" t="n">
-        <v>11</v>
+        <v>22.6</v>
       </c>
       <c r="G90" s="7" t="n">
         <v>1</v>
@@ -5769,28 +5841,28 @@
       <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="n">
-        <v>74</v>
-      </c>
-      <c r="B91" s="6" t="inlineStr">
-        <is>
-          <t>744:485</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D91" s="6" t="n">
+      <c r="A91" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>750:477</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E91" s="6" t="n">
+      <c r="E91" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="F91" s="6" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G91" s="6" t="n">
-        <v>0</v>
+      <c r="F91" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="G91" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H91" s="4" t="n"/>
       <c r="I91" s="4" t="n"/>
@@ -5799,11 +5871,11 @@
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>750:475</t>
+          <t>742:485</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
@@ -5813,10 +5885,10 @@
         <v>3</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>7.8</v>
+        <v>20.6</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>0</v>
@@ -5828,11 +5900,11 @@
     </row>
     <row r="93">
       <c r="A93" s="7" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>738:471</t>
+          <t>750:479</t>
         </is>
       </c>
       <c r="C93" s="7" t="n">
@@ -5842,10 +5914,10 @@
         <v>3</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F93" s="7" t="n">
-        <v>17.6</v>
+        <v>11</v>
       </c>
       <c r="G93" s="7" t="n">
         <v>1</v>
@@ -5856,28 +5928,28 @@
       <c r="K93" s="4" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="B94" s="7" t="inlineStr">
-        <is>
-          <t>736:473</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D94" s="7" t="n">
+      <c r="A94" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>744:485</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E94" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="F94" s="7" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G94" s="7" t="n">
-        <v>1</v>
+      <c r="E94" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G94" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H94" s="4" t="n"/>
       <c r="I94" s="4" t="n"/>
@@ -5886,11 +5958,11 @@
     </row>
     <row r="95">
       <c r="A95" s="6" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>740:485</t>
+          <t>750:475</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
@@ -5903,7 +5975,7 @@
         <v>24</v>
       </c>
       <c r="F95" s="6" t="n">
-        <v>21.9</v>
+        <v>7.8</v>
       </c>
       <c r="G95" s="6" t="n">
         <v>0</v>
@@ -5915,11 +5987,11 @@
     </row>
     <row r="96">
       <c r="A96" s="7" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>748:471</t>
+          <t>738:471</t>
         </is>
       </c>
       <c r="C96" s="7" t="n">
@@ -5929,10 +6001,10 @@
         <v>3</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F96" s="7" t="n">
-        <v>7.6</v>
+        <v>17.6</v>
       </c>
       <c r="G96" s="7" t="n">
         <v>1</v>
@@ -5943,28 +6015,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="n">
-        <v>93</v>
-      </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>750:473</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="6" t="n">
+      <c r="A97" s="7" t="n">
+        <v>89</v>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>736:473</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F97" s="6" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G97" s="6" t="n">
-        <v>0</v>
+      <c r="E97" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="F97" s="7" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G97" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
@@ -5972,28 +6044,28 @@
       <c r="K97" s="4" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="7" t="n">
-        <v>96</v>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>736:471</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D98" s="7" t="n">
+      <c r="A98" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>740:485</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D98" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E98" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="F98" s="7" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="G98" s="7" t="n">
-        <v>1</v>
+      <c r="E98" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F98" s="6" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="G98" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H98" s="4" t="n"/>
       <c r="I98" s="4" t="n"/>
@@ -6002,24 +6074,24 @@
     </row>
     <row r="99">
       <c r="A99" s="7" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>734:477</t>
+          <t>748:471</t>
         </is>
       </c>
       <c r="C99" s="7" t="n">
         <v>2</v>
       </c>
       <c r="D99" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E99" s="7" t="n">
         <v>25</v>
       </c>
       <c r="F99" s="7" t="n">
-        <v>22.8</v>
+        <v>7.6</v>
       </c>
       <c r="G99" s="7" t="n">
         <v>1</v>
@@ -6030,28 +6102,28 @@
       <c r="K99" s="4" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="7" t="n">
-        <v>92</v>
-      </c>
-      <c r="B100" s="7" t="inlineStr">
-        <is>
-          <t>734:479</t>
-        </is>
-      </c>
-      <c r="C100" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E100" s="7" t="n">
+      <c r="A100" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>750:473</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E100" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F100" s="7" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G100" s="7" t="n">
-        <v>1</v>
+      <c r="F100" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G100" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H100" s="4" t="n"/>
       <c r="I100" s="4" t="n"/>
@@ -6059,28 +6131,28 @@
       <c r="K100" s="4" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="7" t="n">
+      <c r="A101" s="6" t="n">
         <v>99</v>
       </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>734:481</t>
-        </is>
-      </c>
-      <c r="C101" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D101" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E101" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="F101" s="7" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="G101" s="7" t="n">
-        <v>1</v>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>750:471</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="F101" s="6" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G101" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H101" s="4" t="n"/>
       <c r="I101" s="4" t="n"/>

</xml_diff>

<commit_message>
Seven banners built (750:483 instead of 750:481), 752:477 added; six to go, all placeable now
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -65,11 +65,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00CDE7C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B9DCF0"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -128,9 +123,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1422,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2784,147 +2776,163 @@
       <c r="J43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>737:483</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="n">
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>748:470</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>738:476</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="n">
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>741:470</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="n"/>
-      <c r="I45" s="4" t="n"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="n">
+      <c r="A46" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>739:456</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="n">
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>745:463</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>6 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>741:470</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="n">
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>750:483</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>9 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="n"/>
-      <c r="I47" s="4" t="n"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J47" s="4" t="n"/>
     </row>
     <row r="48">
@@ -2938,7 +2946,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>745:463</t>
+          <t>737:483</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2956,7 +2964,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Trap 1 site 743:462; 8 slots (file order)</t>
+          <t>5 slots (file order)</t>
         </is>
       </c>
       <c r="H48" s="4" t="n"/>
@@ -2974,7 +2982,7 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>748:470</t>
+          <t>738:463</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2992,7 +3000,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>11 slots (file order)</t>
+          <t>8 slots (file order)</t>
         </is>
       </c>
       <c r="H49" s="4" t="n"/>
@@ -3010,7 +3018,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>750:481</t>
+          <t>738:476</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -3028,7 +3036,7 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>7 slots (file order)</t>
+          <t>11 slots (file order)</t>
         </is>
       </c>
       <c r="H50" s="4" t="n"/>
@@ -3046,7 +3054,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>752:459</t>
+          <t>739:456</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -3064,7 +3072,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>1 slots (file order)</t>
+          <t>10 slots (file order)</t>
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
@@ -3072,35 +3080,35 @@
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>738:463</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>wave 2</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="n">
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>752:459</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>wave 1 complete</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>1 slots (file order)</t>
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
@@ -3108,33 +3116,35 @@
       <c r="J52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
+      <c r="A53" s="7" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="inlineStr"/>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>banner 745:463 (wave 1); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>752:477</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>wave 1</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>nothing (touches today's territory)</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
@@ -3142,31 +3152,31 @@
       <c r="J53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="n">
+      <c r="A54" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
         <is>
           <t>trap</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr"/>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>banner 745:477 (built); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>banner 745:463 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
         <is>
           <t>ring 1 seats: 12</t>
         </is>
@@ -3174,6 +3184,40 @@
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>banner 745:477 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3289,28 +3333,28 @@
       <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>740:461</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="8" t="n">
+      <c r="C3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="7" t="n">
         <v>17.7</v>
       </c>
-      <c r="G3" s="8" t="n">
-        <v>2</v>
+      <c r="G3" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
@@ -3347,28 +3391,28 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>740:463</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8" t="n">
+      <c r="C5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="7" t="n">
         <v>16.8</v>
       </c>
-      <c r="G5" s="8" t="n">
-        <v>2</v>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
@@ -3376,28 +3420,28 @@
       <c r="K5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>746:461</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="n">
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="6" t="n">
         <v>12.7</v>
       </c>
-      <c r="G6" s="7" t="n">
-        <v>1</v>
+      <c r="G6" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
@@ -3405,28 +3449,28 @@
       <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>742:465</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="n">
+      <c r="C7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="6" t="n">
         <v>14.2</v>
       </c>
-      <c r="G7" s="7" t="n">
-        <v>1</v>
+      <c r="G7" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
@@ -3434,28 +3478,28 @@
       <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>740:459</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="8" t="n">
+      <c r="C8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="7" t="n">
         <v>18.7</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>2</v>
+      <c r="G8" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
@@ -3463,28 +3507,28 @@
       <c r="K8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>746:463</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="7" t="n">
+      <c r="C9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="G9" s="7" t="n">
-        <v>1</v>
+      <c r="G9" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
@@ -3492,28 +3536,28 @@
       <c r="K9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>744:465</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="7" t="n">
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="6" t="n">
         <v>12.3</v>
       </c>
-      <c r="G10" s="7" t="n">
-        <v>1</v>
+      <c r="G10" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n"/>
@@ -3550,28 +3594,28 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>740:465</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="8" t="n">
+      <c r="C12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="7" t="n">
         <v>16.1</v>
       </c>
-      <c r="G12" s="8" t="n">
-        <v>2</v>
+      <c r="G12" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
@@ -3579,28 +3623,28 @@
       <c r="K12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>746:465</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="7" t="n">
+      <c r="C13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="F13" s="6" t="n">
         <v>10.5</v>
       </c>
-      <c r="G13" s="7" t="n">
-        <v>1</v>
+      <c r="G13" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
@@ -3637,28 +3681,28 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>738:461</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="8" t="n">
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="7" t="n">
         <v>19.5</v>
       </c>
-      <c r="G15" s="8" t="n">
-        <v>2</v>
+      <c r="G15" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -3724,28 +3768,28 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n">
+      <c r="A18" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>738:459</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="n">
+      <c r="C18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="7" t="n">
         <v>20.4</v>
       </c>
-      <c r="G18" s="8" t="n">
-        <v>2</v>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
@@ -3782,28 +3826,28 @@
       <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>742:467</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="7" t="n">
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="6" t="n">
         <v>13.7</v>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
+      <c r="G20" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -3811,28 +3855,28 @@
       <c r="K20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>748:463</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="7" t="n">
+      <c r="C21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F21" s="7" t="n">
+      <c r="F21" s="6" t="n">
         <v>9.9</v>
       </c>
-      <c r="G21" s="7" t="n">
-        <v>1</v>
+      <c r="G21" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
@@ -3840,28 +3884,28 @@
       <c r="K21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>744:467</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="7" t="n">
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F22" s="6" t="n">
         <v>11.8</v>
       </c>
-      <c r="G22" s="7" t="n">
-        <v>1</v>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
@@ -3869,28 +3913,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>738:465</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="8" t="n">
+      <c r="C23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="7" t="n">
         <v>18.1</v>
       </c>
-      <c r="G23" s="8" t="n">
-        <v>2</v>
+      <c r="G23" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -3927,28 +3971,28 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>740:467</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="7" t="n">
+      <c r="C25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="F25" s="7" t="n">
+      <c r="F25" s="6" t="n">
         <v>15.7</v>
       </c>
-      <c r="G25" s="7" t="n">
-        <v>1</v>
+      <c r="G25" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -3985,28 +4029,28 @@
       <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>748:465</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="7" t="n">
+      <c r="C27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F27" s="7" t="n">
+      <c r="F27" s="6" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="G27" s="7" t="n">
-        <v>1</v>
+      <c r="G27" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -4014,28 +4058,28 @@
       <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>746:467</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="7" t="n">
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="7" t="n">
+      <c r="F28" s="6" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="G28" s="7" t="n">
-        <v>1</v>
+      <c r="G28" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -4072,28 +4116,28 @@
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>738:467</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="7" t="n">
+      <c r="C30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F30" s="7" t="n">
+      <c r="F30" s="6" t="n">
         <v>17.7</v>
       </c>
-      <c r="G30" s="7" t="n">
-        <v>1</v>
+      <c r="G30" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
@@ -4101,28 +4145,28 @@
       <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="6" t="n">
         <v>84</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>748:467</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="7" t="n">
+      <c r="C31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F31" s="7" t="n">
+      <c r="F31" s="6" t="n">
         <v>7.9</v>
       </c>
-      <c r="G31" s="7" t="n">
-        <v>1</v>
+      <c r="G31" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
@@ -4159,28 +4203,28 @@
       <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="n">
+      <c r="A33" s="7" t="n">
         <v>59</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>736:461</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="8" t="n">
+      <c r="C33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="8" t="n">
+      <c r="E33" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="7" t="n">
         <v>21.3</v>
       </c>
-      <c r="G33" s="8" t="n">
-        <v>2</v>
+      <c r="G33" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -4217,28 +4261,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="n">
+      <c r="A35" s="7" t="n">
         <v>62</v>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>736:463</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="8" t="n">
+      <c r="C35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="8" t="n">
+      <c r="E35" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="7" t="n">
         <v>20.6</v>
       </c>
-      <c r="G35" s="8" t="n">
-        <v>2</v>
+      <c r="G35" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -4275,28 +4319,28 @@
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n">
+      <c r="A37" s="7" t="n">
         <v>67</v>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>736:459</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="8" t="n">
+      <c r="C37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="8" t="n">
+      <c r="E37" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="F37" s="8" t="n">
+      <c r="F37" s="7" t="n">
         <v>22.1</v>
       </c>
-      <c r="G37" s="8" t="n">
-        <v>2</v>
+      <c r="G37" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
@@ -4333,28 +4377,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="n">
+      <c r="A39" s="7" t="n">
         <v>74</v>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>736:465</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="8" t="n">
+      <c r="C39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="8" t="n">
+      <c r="E39" s="7" t="n">
         <v>22</v>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F39" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="G39" s="8" t="n">
-        <v>2</v>
+      <c r="G39" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -4391,28 +4435,28 @@
       <c r="K40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="6" t="n">
         <v>78</v>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>742:469</t>
         </is>
       </c>
-      <c r="C41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="7" t="n">
+      <c r="C41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E41" s="7" t="n">
+      <c r="E41" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F41" s="7" t="n">
+      <c r="F41" s="6" t="n">
         <v>13.5</v>
       </c>
-      <c r="G41" s="7" t="n">
-        <v>1</v>
+      <c r="G41" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
@@ -4449,28 +4493,28 @@
       <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="6" t="n">
         <v>82</v>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>744:469</t>
         </is>
       </c>
-      <c r="C43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="7" t="n">
+      <c r="C43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="7" t="n">
+      <c r="E43" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F43" s="7" t="n">
+      <c r="F43" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="G43" s="7" t="n">
-        <v>1</v>
+      <c r="G43" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
@@ -4565,28 +4609,28 @@
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="6" t="n">
         <v>93</v>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>746:469</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="7" t="n">
+      <c r="C47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="7" t="n">
+      <c r="E47" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F47" s="7" t="n">
+      <c r="F47" s="6" t="n">
         <v>9.5</v>
       </c>
-      <c r="G47" s="7" t="n">
-        <v>1</v>
+      <c r="G47" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
@@ -4623,28 +4667,28 @@
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="6" t="n">
         <v>97</v>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>738:469</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="7" t="n">
+      <c r="C49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="7" t="n">
+      <c r="E49" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F49" s="7" t="n">
+      <c r="F49" s="6" t="n">
         <v>17.5</v>
       </c>
-      <c r="G49" s="7" t="n">
-        <v>1</v>
+      <c r="G49" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4" t="n"/>
@@ -5058,28 +5102,28 @@
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="n">
+      <c r="A64" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>742:473</t>
         </is>
       </c>
-      <c r="C64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E64" s="7" t="n">
+      <c r="C64" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F64" s="7" t="n">
+      <c r="F64" s="6" t="n">
         <v>13.9</v>
       </c>
-      <c r="G64" s="7" t="n">
-        <v>1</v>
+      <c r="G64" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
@@ -5116,28 +5160,28 @@
       <c r="K65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="n">
+      <c r="A66" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B66" s="7" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>744:473</t>
         </is>
       </c>
-      <c r="C66" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" s="7" t="n">
+      <c r="C66" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F66" s="7" t="n">
+      <c r="F66" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G66" s="7" t="n">
-        <v>1</v>
+      <c r="G66" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
@@ -5261,28 +5305,28 @@
       <c r="K70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="n">
+      <c r="A71" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>746:473</t>
         </is>
       </c>
-      <c r="C71" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E71" s="7" t="n">
+      <c r="C71" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F71" s="7" t="n">
+      <c r="F71" s="6" t="n">
         <v>10.1</v>
       </c>
-      <c r="G71" s="7" t="n">
-        <v>1</v>
+      <c r="G71" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
@@ -5464,28 +5508,28 @@
       <c r="K77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="7" t="n">
+      <c r="A78" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="B78" s="7" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>748:481</t>
         </is>
       </c>
-      <c r="C78" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D78" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E78" s="7" t="n">
+      <c r="C78" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F78" s="7" t="n">
+      <c r="F78" s="6" t="n">
         <v>13.7</v>
       </c>
-      <c r="G78" s="7" t="n">
-        <v>1</v>
+      <c r="G78" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
@@ -5493,28 +5537,28 @@
       <c r="K78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="7" t="n">
+      <c r="A79" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="B79" s="7" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>746:483</t>
         </is>
       </c>
-      <c r="C79" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D79" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" s="7" t="n">
+      <c r="C79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F79" s="7" t="n">
+      <c r="F79" s="6" t="n">
         <v>16.5</v>
       </c>
-      <c r="G79" s="7" t="n">
-        <v>1</v>
+      <c r="G79" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
@@ -5522,28 +5566,28 @@
       <c r="K79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="n">
+      <c r="A80" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="B80" s="7" t="inlineStr">
+      <c r="B80" s="6" t="inlineStr">
         <is>
           <t>748:473</t>
         </is>
       </c>
-      <c r="C80" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E80" s="7" t="n">
+      <c r="C80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E80" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F80" s="7" t="n">
+      <c r="F80" s="6" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G80" s="7" t="n">
-        <v>1</v>
+      <c r="G80" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n"/>
       <c r="I80" s="4" t="n"/>
@@ -5580,28 +5624,28 @@
       <c r="K81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="7" t="n">
+      <c r="A82" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="B82" s="7" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>748:483</t>
         </is>
       </c>
-      <c r="C82" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E82" s="7" t="n">
+      <c r="C82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F82" s="7" t="n">
+      <c r="F82" s="6" t="n">
         <v>15.4</v>
       </c>
-      <c r="G82" s="7" t="n">
-        <v>1</v>
+      <c r="G82" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
@@ -5609,28 +5653,28 @@
       <c r="K82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="n">
+      <c r="A83" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="B83" s="7" t="inlineStr">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>742:471</t>
         </is>
       </c>
-      <c r="C83" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D83" s="7" t="n">
+      <c r="C83" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E83" s="7" t="n">
+      <c r="E83" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F83" s="7" t="n">
+      <c r="F83" s="6" t="n">
         <v>13.6</v>
       </c>
-      <c r="G83" s="7" t="n">
-        <v>1</v>
+      <c r="G83" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H83" s="4" t="n"/>
       <c r="I83" s="4" t="n"/>
@@ -5667,28 +5711,28 @@
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="n">
+      <c r="A85" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>744:471</t>
         </is>
       </c>
-      <c r="C85" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="7" t="n">
+      <c r="C85" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E85" s="7" t="n">
+      <c r="E85" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F85" s="7" t="n">
+      <c r="F85" s="6" t="n">
         <v>11.6</v>
       </c>
-      <c r="G85" s="7" t="n">
-        <v>1</v>
+      <c r="G85" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
@@ -5725,28 +5769,28 @@
       <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="7" t="n">
+      <c r="A87" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="B87" s="7" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>740:471</t>
         </is>
       </c>
-      <c r="C87" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="7" t="n">
+      <c r="C87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E87" s="7" t="n">
+      <c r="E87" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F87" s="7" t="n">
+      <c r="F87" s="6" t="n">
         <v>15.6</v>
       </c>
-      <c r="G87" s="7" t="n">
-        <v>1</v>
+      <c r="G87" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H87" s="4" t="n"/>
       <c r="I87" s="4" t="n"/>
@@ -5783,28 +5827,28 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="7" t="n">
+      <c r="A89" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>746:471</t>
         </is>
       </c>
-      <c r="C89" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D89" s="7" t="n">
+      <c r="C89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E89" s="7" t="n">
+      <c r="E89" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F89" s="7" t="n">
+      <c r="F89" s="6" t="n">
         <v>9.6</v>
       </c>
-      <c r="G89" s="7" t="n">
-        <v>1</v>
+      <c r="G89" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
@@ -5986,28 +6030,28 @@
       <c r="K95" s="4" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="7" t="n">
+      <c r="A96" s="6" t="n">
         <v>88</v>
       </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>738:471</t>
         </is>
       </c>
-      <c r="C96" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="7" t="n">
+      <c r="C96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="7" t="n">
+      <c r="E96" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="F96" s="7" t="n">
+      <c r="F96" s="6" t="n">
         <v>17.6</v>
       </c>
-      <c r="G96" s="7" t="n">
-        <v>1</v>
+      <c r="G96" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H96" s="4" t="n"/>
       <c r="I96" s="4" t="n"/>
@@ -6073,28 +6117,28 @@
       <c r="K98" s="4" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="7" t="n">
+      <c r="A99" s="6" t="n">
         <v>94</v>
       </c>
-      <c r="B99" s="7" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>748:471</t>
         </is>
       </c>
-      <c r="C99" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" s="7" t="n">
+      <c r="C99" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E99" s="7" t="n">
+      <c r="E99" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F99" s="7" t="n">
+      <c r="F99" s="6" t="n">
         <v>7.6</v>
       </c>
-      <c r="G99" s="7" t="n">
-        <v>1</v>
+      <c r="G99" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H99" s="4" t="n"/>
       <c r="I99" s="4" t="n"/>

</xml_diff>

<commit_message>
20 Sep afternoon: 753:459 and 754:481 dismantled, five banners under construction, 752:477 pending resources
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -1414,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>753:459</t>
+          <t>781:466</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>781:466</t>
+          <t>774:466</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>774:466</t>
+          <t>767:466</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>767:466</t>
+          <t>746:458</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>746:458</t>
+          <t>746:451</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>746:451</t>
+          <t>761:482</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>754:481</t>
+          <t>767:481</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>761:482</t>
+          <t>774:485</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>767:481</t>
+          <t>761:489</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>774:485</t>
+          <t>767:488</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>761:489</t>
+          <t>774:492</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>767:488</t>
+          <t>756:490</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>774:492</t>
+          <t>762:494</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>756:490</t>
+          <t>767:495</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>762:494</t>
+          <t>757:495</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>767:495</t>
+          <t>774:499</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>757:495</t>
+          <t>754:445</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>774:499</t>
+          <t>755:439</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>754:445</t>
+          <t>762:438</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>755:439</t>
+          <t>751:432</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>762:438</t>
+          <t>745:425</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>751:432</t>
+          <t>781:490</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>745:425</t>
+          <t>788:493</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>781:490</t>
+          <t>750:501</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2606,23 +2606,33 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>788:493</t>
+          <t>745:477</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>existing</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr"/>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I39" s="4" t="n"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J39" s="4" t="n"/>
     </row>
     <row r="40">
@@ -2636,23 +2646,33 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>750:501</t>
+          <t>744:480</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>existing</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr"/>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="F40" s="6" t="inlineStr"/>
-      <c r="G40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I40" s="4" t="n"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J40" s="4" t="n"/>
     </row>
     <row r="41">
@@ -2666,7 +2686,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>745:477</t>
+          <t>743:487</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2675,7 +2695,7 @@
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
       <c r="G41" s="6" t="inlineStr">
@@ -2706,7 +2726,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>744:480</t>
+          <t>748:470</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -2715,7 +2735,7 @@
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F42" s="6" t="inlineStr"/>
       <c r="G42" s="6" t="inlineStr">
@@ -2746,7 +2766,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>743:487</t>
+          <t>741:470</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -2755,7 +2775,7 @@
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
       <c r="G43" s="6" t="inlineStr">
@@ -2786,7 +2806,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>748:470</t>
+          <t>745:463</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -2795,7 +2815,7 @@
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F44" s="6" t="inlineStr"/>
       <c r="G44" s="6" t="inlineStr">
@@ -2826,7 +2846,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>741:470</t>
+          <t>750:483</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -2835,7 +2855,7 @@
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
       <c r="G45" s="6" t="inlineStr">
@@ -2866,7 +2886,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>745:463</t>
+          <t>737:483</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -2875,7 +2895,7 @@
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F46" s="6" t="inlineStr"/>
       <c r="G46" s="6" t="inlineStr">
@@ -2906,7 +2926,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>750:483</t>
+          <t>738:463</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -2915,7 +2935,7 @@
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
       <c r="G47" s="6" t="inlineStr">
@@ -2936,111 +2956,123 @@
       <c r="J47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n">
+      <c r="A48" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>737:483</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>5 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>738:476</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>738:463</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>8 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>739:456</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr"/>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>738:476</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>11 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>752:459</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J50" s="4" t="n"/>
     </row>
     <row r="51">
@@ -3054,7 +3086,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>739:456</t>
+          <t>752:477</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -3063,7 +3095,7 @@
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3104,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>10 slots (file order)</t>
+          <t>4 slots (file order)</t>
         </is>
       </c>
       <c r="H51" s="4" t="n"/>
@@ -3080,35 +3112,33 @@
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="n">
+      <c r="A52" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>752:459</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>1 slots (file order)</t>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>743:462</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr"/>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>banner 745:463 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H52" s="4" t="n"/>
@@ -3116,108 +3146,38 @@
       <c r="J52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>banner</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>752:477</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>4 slots (file order)</t>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>743:478</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>trap</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr"/>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>banner 745:477 (built); the old trap's last firing</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>ring 1 seats: 12</t>
         </is>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
       <c r="J53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>743:462</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>banner 745:463 (built); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>743:478</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>trap</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>banner 745:477 (built); the old trap's last firing</t>
-        </is>
-      </c>
-      <c r="G55" s="8" t="inlineStr">
-        <is>
-          <t>ring 1 seats: 12</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3304,28 +3264,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>742:459</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7" t="n">
+      <c r="C2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="6" t="n">
         <v>17.1</v>
       </c>
-      <c r="G2" s="7" t="n">
-        <v>1</v>
+      <c r="G2" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
@@ -3333,28 +3293,28 @@
       <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>740:461</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7" t="n">
+      <c r="C3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F3" s="7" t="n">
+      <c r="F3" s="6" t="n">
         <v>17.7</v>
       </c>
-      <c r="G3" s="7" t="n">
-        <v>1</v>
+      <c r="G3" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
@@ -3391,28 +3351,28 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>740:463</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7" t="n">
+      <c r="C5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="6" t="n">
         <v>16.8</v>
       </c>
-      <c r="G5" s="7" t="n">
-        <v>1</v>
+      <c r="G5" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
@@ -3478,28 +3438,28 @@
       <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>740:459</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="n">
+      <c r="C8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="6" t="n">
         <v>18.7</v>
       </c>
-      <c r="G8" s="7" t="n">
-        <v>1</v>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
@@ -3594,28 +3554,28 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>740:465</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="n">
+      <c r="C12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="6" t="n">
         <v>16.1</v>
       </c>
-      <c r="G12" s="7" t="n">
-        <v>1</v>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
@@ -3652,28 +3612,28 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>742:457</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="7" t="n">
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="6" t="n">
         <v>18.4</v>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>1</v>
+      <c r="G14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
@@ -3681,28 +3641,28 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>738:461</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" s="7" t="n">
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="6" t="n">
         <v>19.5</v>
       </c>
-      <c r="G15" s="7" t="n">
-        <v>1</v>
+      <c r="G15" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -3739,28 +3699,28 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>740:457</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="7" t="n">
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="F17" s="7" t="n">
+      <c r="F17" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="G17" s="7" t="n">
-        <v>1</v>
+      <c r="G17" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -3768,28 +3728,28 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>738:459</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="7" t="n">
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F18" s="6" t="n">
         <v>20.4</v>
       </c>
-      <c r="G18" s="7" t="n">
-        <v>1</v>
+      <c r="G18" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
@@ -3797,28 +3757,28 @@
       <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>748:461</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="7" t="n">
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F19" s="7" t="n">
+      <c r="F19" s="6" t="n">
         <v>11.3</v>
       </c>
-      <c r="G19" s="7" t="n">
-        <v>1</v>
+      <c r="G19" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
@@ -3913,28 +3873,28 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>738:465</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="7" t="n">
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="7" t="n">
+      <c r="F23" s="6" t="n">
         <v>18.1</v>
       </c>
-      <c r="G23" s="7" t="n">
-        <v>1</v>
+      <c r="G23" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -4000,28 +3960,28 @@
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>738:457</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="7" t="n">
+      <c r="C26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F26" s="7" t="n">
+      <c r="F26" s="6" t="n">
         <v>21.5</v>
       </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
+      <c r="G26" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
@@ -4174,28 +4134,28 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>742:455</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="7" t="n">
+      <c r="C32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="7" t="n">
+      <c r="E32" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F32" s="7" t="n">
+      <c r="F32" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="G32" s="7" t="n">
-        <v>1</v>
+      <c r="G32" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -4203,28 +4163,28 @@
       <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>736:461</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="7" t="n">
+      <c r="C33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="7" t="n">
+      <c r="E33" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F33" s="7" t="n">
+      <c r="F33" s="6" t="n">
         <v>21.3</v>
       </c>
-      <c r="G33" s="7" t="n">
-        <v>1</v>
+      <c r="G33" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -4261,28 +4221,28 @@
       <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>736:463</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="7" t="n">
+      <c r="C35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="7" t="n">
+      <c r="E35" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F35" s="7" t="n">
+      <c r="F35" s="6" t="n">
         <v>20.6</v>
       </c>
-      <c r="G35" s="7" t="n">
-        <v>1</v>
+      <c r="G35" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -4290,28 +4250,28 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n">
+      <c r="A36" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>740:455</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="7" t="n">
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F36" s="7" t="n">
+      <c r="F36" s="6" t="n">
         <v>21.2</v>
       </c>
-      <c r="G36" s="7" t="n">
-        <v>1</v>
+      <c r="G36" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="n"/>
@@ -4319,28 +4279,28 @@
       <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="6" t="n">
         <v>67</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>736:459</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="7" t="n">
+      <c r="C37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="7" t="n">
+      <c r="E37" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F37" s="7" t="n">
+      <c r="F37" s="6" t="n">
         <v>22.1</v>
       </c>
-      <c r="G37" s="7" t="n">
-        <v>1</v>
+      <c r="G37" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
@@ -4377,28 +4337,28 @@
       <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>736:465</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="7" t="n">
+      <c r="C39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="7" t="n">
+      <c r="E39" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F39" s="7" t="n">
+      <c r="F39" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G39" s="7" t="n">
-        <v>1</v>
+      <c r="G39" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
@@ -4551,28 +4511,28 @@
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="6" t="n">
         <v>91</v>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>736:457</t>
         </is>
       </c>
-      <c r="C45" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="7" t="n">
+      <c r="C45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="7" t="n">
+      <c r="E45" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="F45" s="7" t="n">
+      <c r="F45" s="6" t="n">
         <v>23.2</v>
       </c>
-      <c r="G45" s="7" t="n">
-        <v>1</v>
+      <c r="G45" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
@@ -4783,28 +4743,28 @@
       <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>740:477</t>
         </is>
       </c>
-      <c r="C53" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="7" t="n">
+      <c r="C53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F53" s="7" t="n">
+      <c r="F53" s="6" t="n">
         <v>17.2</v>
       </c>
-      <c r="G53" s="7" t="n">
-        <v>1</v>
+      <c r="G53" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
@@ -4841,28 +4801,28 @@
       <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n">
+      <c r="A55" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>740:479</t>
         </is>
       </c>
-      <c r="C55" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="7" t="n">
+      <c r="C55" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F55" s="7" t="n">
+      <c r="F55" s="6" t="n">
         <v>18.2</v>
       </c>
-      <c r="G55" s="7" t="n">
-        <v>1</v>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -4899,28 +4859,28 @@
       <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="n">
+      <c r="A57" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>740:475</t>
         </is>
       </c>
-      <c r="C57" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" s="7" t="n">
+      <c r="C57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F57" s="7" t="n">
+      <c r="F57" s="6" t="n">
         <v>16.4</v>
       </c>
-      <c r="G57" s="7" t="n">
-        <v>1</v>
+      <c r="G57" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -5044,28 +5004,28 @@
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="n">
+      <c r="A62" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>740:481</t>
         </is>
       </c>
-      <c r="C62" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="7" t="n">
+      <c r="C62" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F62" s="7" t="n">
+      <c r="F62" s="6" t="n">
         <v>19.3</v>
       </c>
-      <c r="G62" s="7" t="n">
-        <v>1</v>
+      <c r="G62" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
@@ -5131,28 +5091,28 @@
       <c r="K64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="n">
+      <c r="A65" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>738:477</t>
         </is>
       </c>
-      <c r="C65" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="7" t="n">
+      <c r="C65" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F65" s="7" t="n">
+      <c r="F65" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="G65" s="7" t="n">
-        <v>1</v>
+      <c r="G65" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
@@ -5189,28 +5149,28 @@
       <c r="K66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="7" t="n">
+      <c r="A67" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B67" s="7" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>738:479</t>
         </is>
       </c>
-      <c r="C67" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" s="7" t="n">
+      <c r="C67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F67" s="7" t="n">
+      <c r="F67" s="6" t="n">
         <v>19.9</v>
       </c>
-      <c r="G67" s="7" t="n">
-        <v>1</v>
+      <c r="G67" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
@@ -5218,28 +5178,28 @@
       <c r="K67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="n">
+      <c r="A68" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B68" s="7" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>740:473</t>
         </is>
       </c>
-      <c r="C68" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E68" s="7" t="n">
+      <c r="C68" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="F68" s="7" t="n">
+      <c r="F68" s="6" t="n">
         <v>15.9</v>
       </c>
-      <c r="G68" s="7" t="n">
-        <v>1</v>
+      <c r="G68" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
@@ -5392,28 +5352,28 @@
       <c r="K73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="n">
+      <c r="A74" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B74" s="7" t="inlineStr">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>738:481</t>
         </is>
       </c>
-      <c r="C74" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D74" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E74" s="7" t="n">
+      <c r="C74" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E74" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F74" s="7" t="n">
+      <c r="F74" s="6" t="n">
         <v>20.9</v>
       </c>
-      <c r="G74" s="7" t="n">
-        <v>1</v>
+      <c r="G74" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H74" s="4" t="n"/>
       <c r="I74" s="4" t="n"/>
@@ -5450,28 +5410,28 @@
       <c r="K75" s="4" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="7" t="n">
+      <c r="A76" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B76" s="7" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>740:483</t>
         </is>
       </c>
-      <c r="C76" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D76" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E76" s="7" t="n">
+      <c r="C76" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="F76" s="7" t="n">
+      <c r="F76" s="6" t="n">
         <v>20.6</v>
       </c>
-      <c r="G76" s="7" t="n">
-        <v>1</v>
+      <c r="G76" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
@@ -5479,28 +5439,28 @@
       <c r="K76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="7" t="n">
+      <c r="A77" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B77" s="7" t="inlineStr">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>738:473</t>
         </is>
       </c>
-      <c r="C77" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="7" t="n">
+      <c r="C77" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F77" s="7" t="n">
+      <c r="F77" s="6" t="n">
         <v>17.8</v>
       </c>
-      <c r="G77" s="7" t="n">
-        <v>1</v>
+      <c r="G77" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
@@ -5595,28 +5555,28 @@
       <c r="K80" s="4" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="n">
+      <c r="A81" s="6" t="n">
         <v>71</v>
       </c>
-      <c r="B81" s="7" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>738:483</t>
         </is>
       </c>
-      <c r="C81" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D81" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E81" s="7" t="n">
+      <c r="C81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F81" s="7" t="n">
+      <c r="F81" s="6" t="n">
         <v>22.1</v>
       </c>
-      <c r="G81" s="7" t="n">
-        <v>1</v>
+      <c r="G81" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H81" s="4" t="n"/>
       <c r="I81" s="4" t="n"/>
@@ -5682,28 +5642,28 @@
       <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="7" t="n">
+      <c r="A84" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="B84" s="7" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>736:477</t>
         </is>
       </c>
-      <c r="C84" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="7" t="n">
+      <c r="C84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E84" s="7" t="n">
+      <c r="E84" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F84" s="7" t="n">
+      <c r="F84" s="6" t="n">
         <v>20.9</v>
       </c>
-      <c r="G84" s="7" t="n">
-        <v>1</v>
+      <c r="G84" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
@@ -5740,28 +5700,28 @@
       <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="n">
+      <c r="A86" s="6" t="n">
         <v>63</v>
       </c>
-      <c r="B86" s="7" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>736:479</t>
         </is>
       </c>
-      <c r="C86" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="7" t="n">
+      <c r="C86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E86" s="7" t="n">
+      <c r="E86" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F86" s="7" t="n">
+      <c r="F86" s="6" t="n">
         <v>21.7</v>
       </c>
-      <c r="G86" s="7" t="n">
-        <v>1</v>
+      <c r="G86" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -5798,28 +5758,28 @@
       <c r="K87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="7" t="n">
+      <c r="A88" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>736:475</t>
         </is>
       </c>
-      <c r="C88" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="7" t="n">
+      <c r="C88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E88" s="7" t="n">
+      <c r="E88" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F88" s="7" t="n">
+      <c r="F88" s="6" t="n">
         <v>20.3</v>
       </c>
-      <c r="G88" s="7" t="n">
-        <v>1</v>
+      <c r="G88" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H88" s="4" t="n"/>
       <c r="I88" s="4" t="n"/>
@@ -5856,28 +5816,28 @@
       <c r="K89" s="4" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="7" t="n">
+      <c r="A90" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="B90" s="7" t="inlineStr">
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>736:481</t>
         </is>
       </c>
-      <c r="C90" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D90" s="7" t="n">
+      <c r="C90" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E90" s="7" t="n">
+      <c r="E90" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F90" s="7" t="n">
+      <c r="F90" s="6" t="n">
         <v>22.6</v>
       </c>
-      <c r="G90" s="7" t="n">
-        <v>1</v>
+      <c r="G90" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H90" s="4" t="n"/>
       <c r="I90" s="4" t="n"/>
@@ -6059,28 +6019,28 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="7" t="n">
+      <c r="A97" s="6" t="n">
         <v>89</v>
       </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>736:473</t>
         </is>
       </c>
-      <c r="C97" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D97" s="7" t="n">
+      <c r="C97" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E97" s="7" t="n">
+      <c r="E97" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="F97" s="7" t="n">
+      <c r="F97" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="G97" s="7" t="n">
-        <v>1</v>
+      <c r="G97" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>

</xml_diff>

<commit_message>
All 13 banners built; officers page: nodes, traps, banners to take down
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook.xlsx
+++ b/hive_workbook.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,11 +60,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CDE7C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -120,9 +115,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3076,67 +3068,71 @@
       <c r="J50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>752:477</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>wave 1</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="n">
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>nothing (touches today's territory)</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>4 slots (file order)</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
+      <c r="F51" s="6" t="inlineStr"/>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>stands; counted as today's territory</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
       <c r="J51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>Trap 1</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>743:462</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>trap</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr"/>
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>banner 745:463 (built); the old trap's last firing</t>
         </is>
       </c>
-      <c r="G52" s="8" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>ring 1 seats: 12</t>
         </is>
@@ -3146,31 +3142,31 @@
       <c r="J52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="n">
+      <c r="A53" s="7" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>Trap 2</t>
         </is>
       </c>
-      <c r="C53" s="8" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>743:478</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>trap</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr"/>
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>banner 745:477 (built); the old trap's last firing</t>
         </is>
       </c>
-      <c r="G53" s="8" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>ring 1 seats: 12</t>
         </is>
@@ -5207,28 +5203,28 @@
       <c r="K68" s="4" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="n">
+      <c r="A69" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="B69" s="7" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>748:477</t>
         </is>
       </c>
-      <c r="C69" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D69" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E69" s="7" t="n">
+      <c r="C69" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F69" s="7" t="n">
+      <c r="F69" s="6" t="n">
         <v>10.6</v>
       </c>
-      <c r="G69" s="7" t="n">
-        <v>1</v>
+      <c r="G69" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
@@ -5294,28 +5290,28 @@
       <c r="K71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="n">
+      <c r="A72" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>748:479</t>
         </is>
       </c>
-      <c r="C72" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" s="7" t="n">
+      <c r="C72" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F72" s="7" t="n">
+      <c r="F72" s="6" t="n">
         <v>12.1</v>
       </c>
-      <c r="G72" s="7" t="n">
-        <v>1</v>
+      <c r="G72" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
@@ -5845,28 +5841,28 @@
       <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="7" t="n">
+      <c r="A91" s="6" t="n">
         <v>76</v>
       </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>750:477</t>
         </is>
       </c>
-      <c r="C91" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D91" s="7" t="n">
+      <c r="C91" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E91" s="7" t="n">
+      <c r="E91" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F91" s="7" t="n">
+      <c r="F91" s="6" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="G91" s="7" t="n">
-        <v>1</v>
+      <c r="G91" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H91" s="4" t="n"/>
       <c r="I91" s="4" t="n"/>
@@ -5903,28 +5899,28 @@
       <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="7" t="n">
+      <c r="A93" s="6" t="n">
         <v>81</v>
       </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>750:479</t>
         </is>
       </c>
-      <c r="C93" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="7" t="n">
+      <c r="C93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E93" s="7" t="n">
+      <c r="E93" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="F93" s="7" t="n">
+      <c r="F93" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="G93" s="7" t="n">
-        <v>1</v>
+      <c r="G93" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="H93" s="4" t="n"/>
       <c r="I93" s="4" t="n"/>

</xml_diff>